<commit_message>
Created front and back of F letter
Signed-off-by: Student Sofiia Fedchuk (TL_KCOMP_B_Y3) <t00264753@mymtu.ie>
</commit_message>
<xml_diff>
--- a/ComputerGraphics.xlsx
+++ b/ComputerGraphics.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\StudentSofiiaFedchuk\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\StudentSofiiaFedchuk\CGProject\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{207A51C8-9A09-4A06-ABBA-B1181205ACC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0230DC41-B2C6-4D24-9B1C-032F7DB23732}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{84C2E5F2-F3DF-40CE-A751-A48977245F1B}"/>
+    <workbookView xWindow="10830" yWindow="3915" windowWidth="16905" windowHeight="11295" xr2:uid="{84C2E5F2-F3DF-40CE-A751-A48977245F1B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -216,24 +216,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
   </cellXfs>
@@ -268,8 +265,8 @@
       <xdr:row>1</xdr:row>
       <xdr:rowOff>139279</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="5" name="Ink 4">
@@ -288,7 +285,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="5" name="Ink 4">
@@ -333,8 +330,8 @@
       <xdr:row>1</xdr:row>
       <xdr:rowOff>129919</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="6" name="Ink 5">
@@ -353,7 +350,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="6" name="Ink 5">
@@ -398,8 +395,8 @@
       <xdr:row>3</xdr:row>
       <xdr:rowOff>104637</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="7" name="Ink 6">
@@ -418,7 +415,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="7" name="Ink 6">
@@ -463,8 +460,8 @@
       <xdr:row>3</xdr:row>
       <xdr:rowOff>130917</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="8" name="Ink 7">
@@ -483,7 +480,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="8" name="Ink 7">
@@ -528,8 +525,8 @@
       <xdr:row>4</xdr:row>
       <xdr:rowOff>153556</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="13" name="Ink 12">
@@ -548,7 +545,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="13" name="Ink 12">
@@ -593,8 +590,8 @@
       <xdr:row>4</xdr:row>
       <xdr:rowOff>159676</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId11">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="14" name="Ink 13">
@@ -613,7 +610,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="14" name="Ink 13">
@@ -658,8 +655,8 @@
       <xdr:row>6</xdr:row>
       <xdr:rowOff>118915</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId13">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="15" name="Ink 14">
@@ -678,7 +675,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="15" name="Ink 14">
@@ -723,8 +720,8 @@
       <xdr:row>6</xdr:row>
       <xdr:rowOff>125035</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId15">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="18" name="Ink 17">
@@ -743,7 +740,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="18" name="Ink 17">
@@ -784,12 +781,12 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>186720</xdr:colOff>
+      <xdr:colOff>158145</xdr:colOff>
       <xdr:row>10</xdr:row>
       <xdr:rowOff>158351</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId17">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="19" name="Ink 18">
@@ -808,7 +805,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="19" name="Ink 18">
@@ -853,8 +850,8 @@
       <xdr:row>10</xdr:row>
       <xdr:rowOff>156911</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId19">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="22" name="Ink 21">
@@ -873,7 +870,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="22" name="Ink 21">
@@ -918,8 +915,8 @@
       <xdr:row>6</xdr:row>
       <xdr:rowOff>14261</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId21">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="32" name="Ink 31">
@@ -938,7 +935,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="32" name="Ink 31">
@@ -978,13 +975,13 @@
       <xdr:rowOff>167884</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>181034</xdr:colOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>1172</xdr:colOff>
       <xdr:row>8</xdr:row>
       <xdr:rowOff>4735</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId23">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="41" name="Ink 40">
@@ -1003,7 +1000,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="41" name="Ink 40">
@@ -1048,8 +1045,8 @@
       <xdr:row>1</xdr:row>
       <xdr:rowOff>134142</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId25">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="42" name="Ink 41">
@@ -1068,7 +1065,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="42" name="Ink 41">
@@ -1113,8 +1110,8 @@
       <xdr:row>1</xdr:row>
       <xdr:rowOff>101742</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId27">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="43" name="Ink 42">
@@ -1133,7 +1130,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="43" name="Ink 42">
@@ -1178,8 +1175,8 @@
       <xdr:row>3</xdr:row>
       <xdr:rowOff>305</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId29">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="44" name="Ink 43">
@@ -1198,7 +1195,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="44" name="Ink 43">
@@ -1243,8 +1240,8 @@
       <xdr:row>4</xdr:row>
       <xdr:rowOff>149927</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId31">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="45" name="Ink 44">
@@ -1263,7 +1260,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="45" name="Ink 44">
@@ -1308,8 +1305,8 @@
       <xdr:row>4</xdr:row>
       <xdr:rowOff>107807</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId33">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="48" name="Ink 47">
@@ -1328,7 +1325,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="48" name="Ink 47">
@@ -1373,8 +1370,8 @@
       <xdr:row>7</xdr:row>
       <xdr:rowOff>173633</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId35">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="51" name="Ink 50">
@@ -1393,7 +1390,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="51" name="Ink 50">
@@ -1438,8 +1435,8 @@
       <xdr:row>7</xdr:row>
       <xdr:rowOff>119993</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId37">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="52" name="Ink 51">
@@ -1458,7 +1455,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="52" name="Ink 51">
@@ -1503,8 +1500,8 @@
       <xdr:row>9</xdr:row>
       <xdr:rowOff>5596</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId39">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="55" name="Ink 54">
@@ -1523,7 +1520,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="55" name="Ink 54">
@@ -1568,8 +1565,8 @@
       <xdr:row>10</xdr:row>
       <xdr:rowOff>151258</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId41">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="56" name="Ink 55">
@@ -1588,7 +1585,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="56" name="Ink 55">
@@ -1633,8 +1630,8 @@
       <xdr:row>10</xdr:row>
       <xdr:rowOff>139738</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId43">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="59" name="Ink 58">
@@ -1653,7 +1650,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="59" name="Ink 58">
@@ -1698,8 +1695,8 @@
       <xdr:row>18</xdr:row>
       <xdr:rowOff>99752</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId45">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="60" name="Ink 59">
@@ -1718,7 +1715,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="60" name="Ink 59">
@@ -1763,8 +1760,8 @@
       <xdr:row>18</xdr:row>
       <xdr:rowOff>119192</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId47">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="61" name="Ink 60">
@@ -1783,7 +1780,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="61" name="Ink 60">
@@ -1828,8 +1825,8 @@
       <xdr:row>18</xdr:row>
       <xdr:rowOff>122792</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId49">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="64" name="Ink 63">
@@ -1848,7 +1845,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="64" name="Ink 63">
@@ -1893,8 +1890,8 @@
       <xdr:row>10</xdr:row>
       <xdr:rowOff>13018</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId51">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="65" name="Ink 64">
@@ -1913,7 +1910,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="65" name="Ink 64">
@@ -1958,8 +1955,8 @@
       <xdr:row>12</xdr:row>
       <xdr:rowOff>112102</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId53">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="73" name="Ink 72">
@@ -1978,7 +1975,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="73" name="Ink 72">
@@ -2063,8 +2060,8 @@
       <inkml:brushProperty name="height" value="0.025" units="cm"/>
     </inkml:brush>
   </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">61 40 24575,'0'1'0,"-1"0"0,0-1 0,0 1 0,0-1 0,0 1 0,0 0 0,1 0 0,-1 0 0,0-1 0,1 1 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,-1 1 0,1-1 0,0 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,1 2 0,5 34 0,-5-35 0,1 0 0,-1 0 0,0 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,0-1 0,0 1 0,0-1 0,0 1 0,0-1 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,1-1 0,-1 0 0,1 1 0,-1-1 0,1 0 0,-1 0 0,1 0 0,-1 0 0,0-1 0,1 1 0,-1-1 0,1 1 0,-1-1 0,4-1 0,-3-1 0,1 1 0,-1 0 0,1-1 0,-1 1 0,0-1 0,0 0 0,0 0 0,-1 0 0,1-1 0,-1 1 0,1-1 0,-1 1 0,0-1 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1-5 0,-2 7 0,1-1 0,0 1 0,-1-1 0,1 1 0,-1-1 0,0 1 0,0-1 0,0 0 0,0 1 0,-1-1 0,1 1 0,0-1 0,-1 1 0,0-1 0,0 1 0,0-1 0,0 1 0,-1-3 0,-1 3 0,0 1 0,0 0 0,1-1 0,-1 1 0,0 0 0,0 0 0,0 1 0,0-1 0,-1 1 0,1-1 0,0 1 0,0 0 0,0 0 0,0 0 0,-4 1 0,-8-1-89,11 0-17,0-1-1,0 1 1,0 0 0,0 0-1,0 1 1,0-1 0,0 1-1,0 0 1,0 0 0,1 0-1,-5 2 1</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="982.89">206 16 24575,'3'4'0,"-1"0"0,1-1 0,-1 1 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 1 0,-1-1 0,0 0 0,0 1 0,0 6 0,1 61 0,-2-54 0,0-6 0,0 0 0,-1 0 0,0 0 0,-1 0 0,-1 0 0,1 0 0,-2-1 0,-8 22 0,9-29 0,1 0 0,-1 1 0,0-1 0,0-1 0,0 1 0,-1 0 0,1-1 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,-1-1 0,1 0 0,-1 0 0,1 0 0,-1 0 0,0-1 0,1 0 0,-1 0 0,0 0 0,0-1 0,0 1 0,-7-2 0,7 2 0,1-1 0,0 0 0,0 0 0,0-1 0,-1 1 0,1-1 0,0 0 0,0 0 0,0 0 0,0-1 0,0 0 0,1 1 0,-1-1 0,0 0 0,-4-4 0,5 2 0,0 1 0,1-1 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1 0 0,0-1 0,0 1 0,0-1 0,0 1 0,0-6 0,0-2-1365,1 2-5461</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">40 40 24575,'0'1'0,"-1"0"0,0-1 0,1 1 0,-1-1 0,0 1 0,1 0 0,0 0 0,-1 0 0,1-1 0,0 1 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,-1 1 0,1-1 0,0 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,1 2 0,2 34 0,-2-35 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1-1 0,-1 1 0,0-1 0,0 1 0,1-1 0,-1 0 0,0 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1-1 0,-1 0 0,1 1 0,-1-1 0,1 0 0,0 0 0,0 0 0,-1 0 0,0-1 0,1 1 0,-1-1 0,1 1 0,0-1 0,1-1 0,-1-1 0,1 1 0,-1 0 0,1-1 0,-2 1 0,1-1 0,0 0 0,0 0 0,0 0 0,-1-1 0,1 1 0,0-1 0,-1 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0-5 0,-1 7 0,1-1 0,-1 1 0,0-1 0,1 1 0,-1-1 0,0 1 0,0-1 0,0 0 0,0 1 0,-1-1 0,1 1 0,0-1 0,0 1 0,-1-1 0,0 1 0,1-1 0,-1 1 0,0-3 0,-1 3 0,0 1 0,0 0 0,1-1 0,-1 1 0,0 0 0,0 0 0,0 1 0,0-1 0,0 1 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,-3 1 0,-4-1-89,6 0-17,1-1-1,-1 1 1,0 0 0,1 0-1,-1 1 1,1-1 0,-1 1-1,0 0 1,1 0 0,0 0-1,-3 2 1</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="982.89">133 16 24575,'2'4'0,"-1"0"0,1-1 0,0 1 0,-1 0 0,0 0 0,1 0 0,-2 0 0,1 1 0,0-1 0,0 0 0,-1 1 0,1 6 0,0 61 0,-1-54 0,0-6 0,0 1 0,0-1 0,-1 0 0,0 0 0,-1 0 0,1 0 0,-2-1 0,-5 22 0,6-29 0,1 0 0,-1 1 0,0-1 0,0-1 0,0 1 0,0 0 0,0-1 0,-1 0 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1-1 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 0 0,0 0 0,0 0 0,0-1 0,-1 1 0,-3-2 0,3 2 0,2-1 0,-1 0 0,1 0 0,-1-1 0,0 1 0,0-1 0,1 0 0,-1 0 0,0 0 0,1-1 0,-1 0 0,1 1 0,0-1 0,-1 0 0,-2-4 0,3 2 0,0 1 0,1-1 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 0 0,0-1 0,1 1 0,-1-1 0,0 1 0,1-6 0,-1-2-1365,1 2-5461</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -2118,14 +2115,14 @@
       <inkml:brushProperty name="height" value="0.025" units="cm"/>
     </inkml:brush>
   </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">32 72 24575,'-5'-3'0,"11"-2"0,-2-1 0,-4 6 0,0 0 0,1 0 0,-1 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,-1-1 0,1 1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,18-2 0,-16 2 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 1 0,-1-1 0,1 0 0,-1 0 0,1 1 0,-1-1 0,1 0 0,-1 1 0,1-1 0,-1 1 0,1-1 0,-1 0 0,0 1 0,1-1 0,-1 1 0,0-1 0,1 1 0,-1-1 0,0 1 0,0 0 0,1-1 0,-1 1 0,0-1 0,0 1 0,0 0 0,0-1 0,0 1 0,0-1 0,0 1 0,0 0 0,0-1 0,0 1 0,0-1 0,0 1 0,0 0 0,0-1 0,-1 1 0,1-1 0,0 1 0,0-1 0,-1 1 0,1-1 0,0 1 0,-1-1 0,1 1 0,-1-1 0,1 1 0,0-1 0,-2 1 0,2 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0-1 0,0 1 0,0 0 0,0-1 0,0 0 0,0 1 0,0-1 0,0 1 0,0-1 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0-1 0,0 1 0,-1-1 0,1 1 0,0-1 0,0 0 0,0 1 0,1-1 0,-1 0 0,-2-1 0,2 0 0,0 1 0,0 0 0,0-1 0,0 1 0,0-1 0,0 1 0,0-1 0,0 1 0,1-1 0,-1 0 0,1 1 0,-1-1 0,1 0 0,0 0 0,-1 1 0,1-1 0,0 0 0,0 0 0,0 1 0,0-1 0,1 0 0,-1 0 0,0 1 0,1-1 0,-1 0 0,1 1 0,1-4 0,-1 3 0,0 1 0,-1-1 0,1 0 0,0 1 0,1-1 0,-1 1 0,0-1 0,0 1 0,1 0 0,-1-1 0,0 1 0,1 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 1 0,0-1 0,-1 1 0,1-1 0,0 1 0,0-1 0,3 1 0,-4 1 0,0-1 0,1 1 0,-1-1 0,0 1 0,0 0 0,0 0 0,1 0 0,-1 0 0,0-1 0,0 1 0,-1 1 0,1-1 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 1 0,0-1 0,-1 0 0,0 1 0,1-1 0,-1 0 0,0 1 0,1-1 0,-1 1 0,0-1 0,0 0 0,0 1 0,0-1 0,0 1 0,0-1 0,-1 0 0,0 3 0,1-2-114,0 0 1,-1 0-1,1 0 0,-1 0 0,0 0 1,1 0-1,-1 0 0,0 0 0,0 0 1,0 0-1,-3 2 0,1 0-6712</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="966.59">45 272 24575,'-16'72'0,"16"-70"0,-25 118 0,23-107 0,1 1 0,0 0 0,1 0 0,1 0 0,0 0 0,5 25 0,-5-36-1,1 1 1,-1-1-1,1 0 0,-1 1 0,1-1 0,0 0 0,1 0 0,-1 0 1,0-1-1,1 1 0,-1 0 0,1-1 0,0 0 0,0 0 1,0 1-1,0-2 0,0 1 0,1 0 0,-1-1 0,0 1 0,5 0 1,22 13-1347,-23-11-5479</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="2119.56">201 445 24575,'-1'29'0,"0"-12"0,1 1 0,1 0 0,2 17 0,-2-31 0,-1-1 0,1 1 0,0-1 0,0 1 0,0-1 0,0 1 0,1-1 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1-1 0,-1 1 0,1-1 0,0 0 0,0 1 0,4 1 0,-6-3 0,0-1 0,0 1 0,0-1 0,-1 1 0,1-1 0,0 0 0,0 0 0,0 1 0,0-1 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,-1-1 0,1 1 0,0 0 0,0 0 0,0-1 0,0 1 0,-1 0 0,1-1 0,0 1 0,0-1 0,-1 1 0,1-1 0,0 0 0,-1 1 0,2-2 0,-1 0 0,0-1 0,1 1 0,-1-1 0,0 0 0,0 0 0,0 1 0,-1-1 0,1 0 0,-1 0 0,1-4 0,-1-5 0,0 0 0,0 0 0,-1 0 0,-3-15 0,2 24-82,1-1 0,0 0-1,-1 1 1,0-1 0,0 1 0,0 0-1,0 0 1,-1 0 0,-4-5 0,4 5-461,-2-3-6283</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="2704.65">384 685 24575,'0'4'0,"0"5"0,0 2 0,0 2 0,0 0 0,0 1 0,0 3 0,-2 0 0,-3 0 0,-1-1 0,1-3-8191</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="4125.85">580 578 24575,'-1'1'0,"0"-1"0,0 1 0,0 0 0,1-1 0,-1 1 0,0 0 0,0 0 0,1 0 0,-1 0 0,0-1 0,1 1 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,0 1 0,0-1 0,0 0 0,-1 0 0,1 0 0,0 0 0,1 0 0,-1 0 0,0 1 0,1 33 0,10 12 0,-10-45 0,-1-1 0,1 1 0,-1 0 0,1 0 0,0 0 0,-1-1 0,1 1 0,0 0 0,0-1 0,0 1 0,0-1 0,1 1 0,-1-1 0,0 1 0,1-1 0,-1 0 0,1 0 0,-1 1 0,1-1 0,-1 0 0,3 1 0,-2-3 0,-1 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0-1 0,-1 1 0,1 0 0,0 0 0,-1-1 0,1 1 0,0-1 0,-1 1 0,1-1 0,-1 1 0,0-1 0,0 1 0,1-1 0,-1-1 0,5-37 0,-5 28-45,-1 1-1,0 0 0,-1 0 1,0 0-1,-1 0 0,0 0 1,-7-14-1,3 5-954,3 7-5826</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="4648.87">698 778 24575,'0'2'0,"0"4"0,0 2 0,0 2 0,2 0 0,1 0 0,0 1 0,-1 1 0,-1 0 0,0 1 0,0 0 0,-1 0 0,0 1 0,0-1 0,-2-2 0,-1-3-8191</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="5579.42">802 672 24575,'1'0'0,"0"1"0,-1 0 0,1-1 0,0 1 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 2 0,3 28 0,-3-29 0,0 31 0,1 25 0,0-55 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,1 0 0,0-1 0,0 1 0,4 4 0,-6-6 0,1-1 0,0 0 0,-1 0 0,1 1 0,0-1 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,-1-1 0,1 1 0,0 0 0,-1-1 0,1 1 0,0-1 0,-1 1 0,1 0 0,0-1 0,-1 1 0,1-1 0,-1 0 0,1 1 0,-1-1 0,1 1 0,-1-1 0,0 0 0,1 1 0,-1-1 0,0 0 0,1 0 0,-1-1 0,18-36 0,-16 34 0,1-3-85,-1 1 0,0-1-1,0 0 1,-1 0 0,1 0-1,-2 0 1,1 1 0,-1-1-1,0 0 1,0 0 0,-1 0-1,0 0 1,0 0 0,-1 0-1,-3-11 1,-1 5-6741</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="6561.15">959 565 24575,'0'22'0,"1"1"0,1-1 0,1 0 0,1 1 0,13 39 0,-12-44 0,-1 0 0,-1 1 0,-1-1 0,0 1 0,-1-1 0,-1 1 0,-1-1 0,-5 33 0,2-40-136,-1 0-1,1 0 1,-2 0-1,1-1 1,-2 0-1,1 0 1,-1-1-1,0 1 0,-10 8 1,9-9-6690</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">28 78 24575,'-4'-3'0,"9"-3"0,-2 0 0,-3 6 0,0 0 0,1 0 0,-1 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0-2 0,0 2 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,-1-1 0,1 1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,15-2 0,-13 2 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,1 0 0,0 1 0,-1-1 0,1 0 0,-1 0 0,1 1 0,-1-1 0,1 0 0,-1 1 0,1-1 0,-1 1 0,1-1 0,-1 0 0,0 1 0,0-1 0,0 2 0,0-2 0,1 1 0,-1-1 0,0 1 0,0 0 0,1-1 0,-1 1 0,0-1 0,0 1 0,0 0 0,0-1 0,0 1 0,0-1 0,0 1 0,0 0 0,0-1 0,0 1 0,0-1 0,0 1 0,0 1 0,0-2 0,-1 1 0,1-1 0,0 1 0,0-1 0,-1 1 0,1-1 0,0 1 0,0-1 0,0 1 0,-1-1 0,1 1 0,0-1 0,-2 1 0,2 0 0,-1 0 0,0 0 0,0 0 0,0 1 0,1-2 0,-1 1 0,0 0 0,0-1 0,0 1 0,0 0 0,0-1 0,0 0 0,1 1 0,-1-1 0,0 1 0,0-1 0,-1 0 0,1 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,1-1 0,-1 1 0,0 0 0,0-1 0,0 1 0,-1-1 0,1 1 0,1-1 0,-1 0 0,0 1 0,1-1 0,-1-1 0,-2 0 0,2 0 0,1 1 0,-1 0 0,0-1 0,0 1 0,0-1 0,0 0 0,0 0 0,0 1 0,1-1 0,0 0 0,0 1 0,-1-1 0,1-1 0,0 1 0,-1 1 0,1-1 0,0 0 0,0 0 0,0 1 0,0-2 0,1 1 0,-1 0 0,0 1 0,1-1 0,-1 0 0,0 1 0,2-5 0,-1 4 0,0 1 0,-1-1 0,1 0 0,0 1 0,0-2 0,0 2 0,0-1 0,0 1 0,1 0 0,-1-1 0,0 1 0,0 0 0,1 0 0,-1-1 0,1 1 0,-1 0 0,0 0 0,1 1 0,0-1 0,-1 1 0,0-1 0,1 1 0,0-1 0,2 1 0,-3 1 0,0-1 0,1 1 0,-1-1 0,-1 1 0,1 0 0,0 0 0,1 0 0,-1 1 0,0-2 0,0 1 0,-1 1 0,0-1 0,1 0 0,0 0 0,0 0 0,-1 0 0,1 1 0,0-1 0,-1 1 0,0 0 0,1-1 0,-1 0 0,0 1 0,1-1 0,-1 1 0,0-1 0,0 0 0,0 2 0,0-2 0,0 1 0,0-1 0,-1 0 0,0 3 0,1-1-114,0-1 1,-1 0-1,1 0 0,-1 0 0,0 0 1,1 1-1,-1-1 0,0 0 0,1 0 1,-1 0-1,-3 3 0,2-1-6712</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="966.59">39 295 24575,'-14'78'0,"14"-76"0,-22 128 0,21-116 0,0 1 0,0 0 0,1 0 0,1 0 0,0 1 0,4 26 0,-4-39-1,1 1 1,-2 0-1,2-1 0,-1 1 0,1 0 0,0-1 0,0 0 0,0 0 1,0-1-1,0 2 0,0-1 0,1-1 0,-1 0 0,1 0 1,0 2-1,-1-3 0,1 1 0,0 0 0,0-1 0,-1 1 0,5 1 1,20 13-1347,-21-12-5479</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="2119.56">175 482 24575,'0'31'0,"-1"-12"0,1 0 0,1 1 0,1 18 0,-1-34 0,-1-1 0,1 2 0,0-2 0,0 1 0,-1-1 0,1 2 0,1-2 0,-1 0 0,1 1 0,-1-1 0,1 0 0,0 0 0,0 1 0,-1-1 0,2-1 0,-1 1 0,0-1 0,1 1 0,0 0 0,3 1 0,-5-3 0,0-1 0,-1 1 0,1-1 0,-1 1 0,1-1 0,0 0 0,0 0 0,0 1 0,0-1 0,-1 0 0,0 0 0,1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,-1-1 0,1 1 0,-1 0 0,1 0 0,0-1 0,0 1 0,-1 0 0,1-1 0,0 1 0,0-1 0,-1 1 0,1-1 0,-1 0 0,0 1 0,2-2 0,-1 0 0,0-2 0,1 2 0,-1-1 0,-1 0 0,1-1 0,0 2 0,-1-1 0,1 0 0,-1 0 0,1-5 0,-1-5 0,0 0 0,0 0 0,-1 0 0,-2-16 0,1 25-82,1 0 0,0 0-1,-1 1 1,1-2 0,-1 2 0,0 0-1,0-1 1,0 1 0,-4-5 0,3 4-461,-1-2-6283</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="2704.65">335 742 24575,'0'4'0,"0"6"0,0 2 0,0 2 0,0 0 0,0 1 0,0 4 0,-2-1 0,-2 1 0,-1-2 0,0-3-8191</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="4125.85">506 626 24575,'-1'1'0,"0"-1"0,0 1 0,1 0 0,0-1 0,-1 1 0,0 0 0,0 1 0,1-1 0,-1 0 0,0-1 0,1 1 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 0 0,0 2 0,0-2 0,0 0 0,-1 0 0,1 0 0,0 0 0,1 0 0,-1 0 0,0 1 0,0 36 0,10 13 0,-9-49 0,-1-1 0,1 2 0,-1-1 0,1 0 0,0 0 0,-1-1 0,0 1 0,1 0 0,0 0 0,0 0 0,0-1 0,1 1 0,-1-1 0,-1 1 0,2-1 0,-1 0 0,1 0 0,-1 2 0,0-2 0,0 0 0,3 1 0,-3-3 0,0 0 0,0 0 0,0 0 0,0 0 0,1-1 0,-1 1 0,-1 0 0,1 0 0,0 0 0,0-1 0,-1 1 0,1 0 0,0 0 0,-1-1 0,1 0 0,0 0 0,-1 1 0,0-1 0,0 1 0,0-1 0,0 1 0,1-1 0,-1-2 0,5-39 0,-5 30-45,-1 1-1,0 0 0,-1 0 1,0 0-1,0 0 0,-1 0 1,-6-15-1,3 6-954,3 7-5826</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="4648.87">609 843 24575,'0'2'0,"0"4"0,0 3 0,0 2 0,2 0 0,0 0 0,1 0 0,-1 2 0,-1 0 0,-1 2 0,1-1 0,-1 0 0,0 1 0,0-1 0,-1-2 0,-2-3-8191</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="5579.42">700 728 24575,'1'0'0,"-1"1"0,0 0 0,1-1 0,0 1 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 1 0,-1-1 0,0 0 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 3 0,2 29 0,-2-31 0,0 34 0,1 27 0,0-60 0,-1 0 0,1 1 0,-1-1 0,1 0 0,0 0 0,-1 1 0,2-1 0,-1 0 0,0 0 0,1 1 0,-1-2 0,1 1 0,3 5 0,-5-7 0,1-1 0,0 0 0,-1 0 0,1 1 0,0-1 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,0 0 0,1 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,-1-1 0,1 1 0,-1 0 0,0-1 0,1 1 0,0-1 0,-1 1 0,1 0 0,0-1 0,-1 1 0,1-2 0,-1 1 0,1 1 0,-1-1 0,0 1 0,0-1 0,0 0 0,1 1 0,-1-1 0,0 0 0,1 0 0,-1-1 0,16-39 0,-14 36 0,0-2-85,0 0 0,0 0-1,0-1 1,-2 0 0,2 1-1,-2-1 1,1 2 0,-1-2-1,0 1 1,0-1 0,-1 0-1,0 1 1,0-1 0,0 1-1,-4-13 1,0 6-6741</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="6561.15">837 612 24575,'0'24'0,"1"1"0,0-1 0,2-1 0,0 2 0,12 42 0,-10-47 0,-2-1 0,0 2 0,-1-1 0,-1 0 0,0 0 0,-1 0 0,-1 0 0,-4 35 0,2-43-136,-2 0-1,2 0 1,-3 0-1,2-2 1,-2 1-1,1 0 1,-1-1-1,0 1 0,-9 8 1,8-9-6690</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -2152,7 +2149,7 @@
       <inkml:brushProperty name="height" value="0.025" units="cm"/>
     </inkml:brush>
   </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">0 124 24575,'0'6'0,"0"-1"0,1 1 0,-1 0 0,1 0 0,0-1 0,0 1 0,1-1 0,0 1 0,0-1 0,0 0 0,5 9 0,-5-12 0,0 1 0,1-1 0,-1 1 0,0-1 0,1 0 0,-1 0 0,1 0 0,-1-1 0,1 1 0,0 0 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,1 1 0,-1-1 0,0 0 0,0 0 0,6 0 0,-7 0 0,1-1 0,0 1 0,-1 0 0,1-1 0,-1 0 0,1 0 0,-1 1 0,1-1 0,-1-1 0,0 1 0,1 0 0,-1-1 0,0 1 0,0-1 0,0 1 0,0-1 0,0 0 0,0 0 0,-1 0 0,3-3 0,-2 0 0,1 1 0,-1-1 0,0 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,0-1 0,0-9 0,-1 6 0,0 1 0,0-1 0,-1 1 0,0-1 0,0 1 0,-1 0 0,0-1 0,-1 1 0,0 0 0,0 0 0,0 1 0,-10-15 0,12 20-7,0 1-1,-1-1 0,1 1 0,0-1 1,-1 1-1,0-1 0,1 1 0,-1 0 1,0 0-1,0 0 0,1 0 1,-1 0-1,-3-1 0,5 2 15,-1 0-1,0 0 0,0 0 1,1 0-1,-1 0 1,0 0-1,0 0 0,1 0 1,-1 1-1,0-1 1,0 0-1,1 0 0,-1 1 1,0-1-1,1 1 1,-1-1-1,0 0 0,1 1 1,-1-1-1,1 1 0,-1-1 1,1 1-1,-1 0 1,0 0-1,-2 5-49,-1 0 1,1 1-1,1-1 0,-1 1 1,1-1-1,-1 10 0,-5 9-1075,5-15-5708</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">0 124 24575,'0'6'0,"0"-1"0,1 1 0,-1 0 0,1 0 0,-1-1 0,1 1 0,1-1 0,-1 1 0,1-1 0,-1 0 0,5 9 0,-5-12 0,1 1 0,0-1 0,0 1 0,-1-1 0,2 0 0,-2 0 0,1 0 0,0-1 0,0 1 0,1 0 0,-1-1 0,0 0 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1-1 0,1 1 0,-1-1 0,1 0 0,-1 0 0,5 0 0,-5 0 0,0-1 0,0 1 0,0 0 0,0-1 0,0 0 0,0 0 0,0 1 0,0-1 0,-1-1 0,1 1 0,0 0 0,0-1 0,-1 1 0,1-1 0,0 1 0,-1-1 0,1 0 0,-1 0 0,0 0 0,2-3 0,-1 0 0,0 1 0,-1-1 0,1 0 0,0 0 0,-2 0 0,2 0 0,-1 0 0,-1-1 0,1-9 0,-1 6 0,0 1 0,0-1 0,-1 1 0,1-1 0,-1 1 0,-1 0 0,1-1 0,-2 1 0,1 0 0,0 0 0,-1 1 0,-7-15 0,10 20-7,-1 1-1,-1-1 0,2 1 0,-1-1 1,-1 1-1,1-1 0,0 1 0,-1 0 1,1 0-1,-1 0 0,1 0 1,0 0-1,-3-1 0,4 2 15,-1 0-1,0 0 0,1 0 1,0 0-1,-1 0 1,0 0-1,0 0 0,1 0 1,0 1-1,-1-1 1,0 0-1,1 0 0,-1 1 1,0-1-1,1 1 1,0-1-1,-1 0 0,1 1 1,-1-1-1,1 1 0,-1-1 1,1 1-1,0 0 1,-1 0-1,-1 5-49,-2 0 1,2 1-1,1-1 0,-2 1 1,2-1-1,-2 10 0,-3 9-1075,4-15-5708</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -2179,7 +2176,7 @@
       <inkml:brushProperty name="height" value="0.025" units="cm"/>
     </inkml:brush>
   </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">0 161 24575,'2'-5'0,"0"0"0,0 0 0,1 0 0,-1 1 0,1-1 0,0 1 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 1 0,6-4 0,8-9 0,-8 4 0,-1 1 0,0-2 0,0 1 0,9-21 0,-18 33 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,1 1 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,4 18 0,-1 21 0,-11 77 134,0-23-1633,7-80-5327</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">0 161 24575,'1'-5'0,"0"0"0,0 0 0,1 0 0,-1 1 0,1-1 0,-1 1 0,2 0 0,-2 0 0,1 0 0,0 0 0,0 0 0,1 1 0,2-4 0,5-9 0,-5 4 0,0 1 0,0-2 0,0 1 0,5-21 0,-10 33 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,1 1 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,2 18 0,-1 21 0,-5 77 134,0-23-1633,3-80-5327</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -2206,7 +2203,7 @@
       <inkml:brushProperty name="height" value="0.025" units="cm"/>
     </inkml:brush>
   </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">37 14 24575,'41'-6'0,"-35"4"0,0 0 0,0 1 0,0 0 0,1 0 0,-1 1 0,0 0 0,9 1 0,-14-1 0,1 1 0,0-1 0,0 1 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,-1 1 0,1-1 0,-1 0 0,1 1 0,-1-1 0,0 1 0,0 0 0,0-1 0,0 1 0,0 0 0,0-1 0,0 1 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,0 0 0,1 3 0,-1 1 0,0 0 0,0 0 0,0 1 0,0-1 0,-1 0 0,0 0 0,0 0 0,-1 1 0,0-1 0,0-1 0,0 1 0,-1 0 0,0-1 0,0 1 0,0-1 0,-1 0 0,-8 9 0,4-5 0,0 0 0,-1-1 0,-1 0 0,1 0 0,-1-1 0,0-1 0,-1 0 0,-13 7 0,14-10 0,-12 8 0,24-7 0,14-3 0,177-2-1365,-178 1-5461</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">37 15 24575,'41'-6'0,"-35"4"0,0-1 0,0 2 0,0 0 0,1 0 0,-1 1 0,0 0 0,9 1 0,-14-1 0,1 1 0,0-1 0,0 1 0,0 0 0,-1 1 0,1-1 0,0 0 0,-1 0 0,1 0 0,-1 1 0,1-1 0,-1 0 0,1 2 0,-1-2 0,0 1 0,0 0 0,0-1 0,0 2 0,0-1 0,0-1 0,0 1 0,-1 0 0,1 1 0,-1-1 0,1 0 0,-1 0 0,0 0 0,1 4 0,-1 1 0,0-1 0,0 1 0,0 1 0,0-2 0,-1 1 0,0 0 0,0-1 0,-1 2 0,0-1 0,0-2 0,0 2 0,-1 0 0,0-2 0,0 2 0,0-2 0,-1 1 0,-8 10 0,4-6 0,0 0 0,-1-2 0,-1 1 0,1 0 0,-1-1 0,0-1 0,-1-1 0,-13 9 0,14-12 0,-12 9 0,24-7 0,14-4 0,177-2-1365,-178 1-5461</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -2233,7 +2230,7 @@
       <inkml:brushProperty name="height" value="0.025" units="cm"/>
     </inkml:brush>
   </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">0 59 24575,'6'-4'0,"0"0"0,1 0 0,-1 0 0,1 1 0,-1 0 0,11-3 0,15-8 0,-28 11 0,-1 1 0,1 0 0,0 0 0,1 1 0,-1-1 0,0 1 0,0 0 0,1 0 0,-1 1 0,0-1 0,1 1 0,-1 0 0,1 0 0,-1 0 0,0 1 0,1-1 0,-1 1 0,0 0 0,8 3 0,-8-2 0,-1 0 0,0 0 0,0 0 0,-1 0 0,1 1 0,0-1 0,-1 1 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,-1 1 0,1-1 0,-1 0 0,0 1 0,0-1 0,-1 1 0,1 0 0,-1-1 0,0 1 0,0 5 0,0-6 0,0 0 0,-1-1 0,1 1 0,-1 0 0,0-1 0,0 1 0,0-1 0,0 1 0,0-1 0,0 0 0,0 1 0,-1-1 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0-1 0,0 0 0,-1 1 0,1-1 0,-1 0 0,1 0 0,-3 1 0,-25 16 0,30-18 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,1 1 0,14 5 0,18 1 0,30 0 0,-45-7 0,1 2 0,-1 0 0,0 1 0,0 1 0,-1 0 0,1 2 0,25 11 0,-41-17 0,0 1 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,1 1 0,-1-1 0,1 0 0,-1 1 0,0 0 0,0-1 0,0 1 0,0-1 0,0 1 0,0 0 0,0 0 0,-1 0 0,1 0 0,0-1 0,-1 1 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,0-1 0,-1 3 0,0 0 0,-1 0 0,0-1 0,0 1 0,0-1 0,0 0 0,0 0 0,-1 0 0,1 0 0,-1-1 0,0 1 0,0-1 0,0 0 0,0 0 0,0-1 0,-7 3 0,-21 2-273,-1 0 0,0-3 0,0 0 0,-36-3 0,57 0-6553</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">0 59 24575,'5'-4'0,"0"0"0,1 0 0,-1 0 0,1 1 0,-1 0 0,9-3 0,12-8 0,-22 11 0,-2 1 0,2 0 0,-1 0 0,1 1 0,-1-1 0,1 1 0,-1 0 0,1 0 0,0 1 0,-1-1 0,1 1 0,-1 0 0,2 0 0,-2 0 0,0 1 0,1-1 0,0 1 0,-1 0 0,7 3 0,-7-2 0,0 0 0,-1 0 0,1 0 0,-1 0 0,0 1 0,1-1 0,-2 1 0,2 0 0,-2 0 0,1 0 0,0 0 0,-1 0 0,0 0 0,1 0 0,-1 1 0,0-1 0,0 0 0,0 1 0,0-1 0,-1 1 0,1 0 0,-1-1 0,0 1 0,0 5 0,0-6 0,0 0 0,-1-1 0,1 1 0,-1 0 0,0-1 0,0 1 0,1-1 0,-1 1 0,0-1 0,0 0 0,0 1 0,0-1 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,0-1 0,1 1 0,-1 0 0,0-1 0,1 0 0,-2 1 0,2-1 0,-2 0 0,1 0 0,-2 1 0,-21 16 0,25-18 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,1 1 0,12 5 0,14 1 0,26 0 0,-38-7 0,0 2 0,0 0 0,0 1 0,0 1 0,0 0 0,0 2 0,20 11 0,-33-17 0,0 1 0,-1 0 0,0 0 0,1 0 0,0 0 0,-2 0 0,2 0 0,-1 0 0,1 1 0,-2-1 0,2 0 0,-1 1 0,0 0 0,0-1 0,-1 1 0,1-1 0,0 1 0,0 0 0,0 0 0,-1 0 0,1 0 0,-1-1 0,0 1 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,0-1 0,-1 3 0,1 0 0,-2 0 0,1-1 0,-1 1 0,1-1 0,-1 0 0,1 0 0,-2 0 0,2 0 0,-2-1 0,1 1 0,0-1 0,-1 0 0,1 0 0,0-1 0,-6 3 0,-18 2-273,-1 0 0,1-3 0,-1 0 0,-29-3 0,47 0-6553</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -2288,8 +2285,8 @@
       <inkml:brushProperty name="height" value="0.025" units="cm"/>
     </inkml:brush>
   </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">71 102 24575,'-3'2'0,"0"0"0,0 0 0,0 0 0,0 1 0,1-1 0,-1 1 0,1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,-2 5 0,3-6 0,-2 4 0,-2 2 0,0 1 0,1-1 0,0 1 0,0 0 0,-3 15 0,6-22 0,1-1 0,0 1 0,0 0 0,0-1 0,0 1 0,0-1 0,0 1 0,0 0 0,1-1 0,-1 1 0,0-1 0,1 1 0,-1-1 0,1 1 0,0-1 0,0 1 0,-1-1 0,1 0 0,0 1 0,0-1 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 1 0,0-2 0,1 1 0,-1 0 0,0 0 0,1 0 0,-1-1 0,1 1 0,-1-1 0,1 1 0,-1-1 0,1 1 0,0-1 0,-1 0 0,1 0 0,1 0 0,23 3 0,0-2 0,-1 0 0,30-4 0,-31 1 0,0 1 0,1 1 0,39 5 0,-61-5 0,-1 1 0,1-1 0,-1 0 0,1 1 0,-1 0 0,0-1 0,1 1 0,-1 0 0,0 0 0,1 0 0,-1 1 0,0-1 0,0 0 0,0 1 0,0-1 0,-1 1 0,1 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,-1 1 0,1-1 0,-1 1 0,1-1 0,-1 0 0,0 1 0,0-1 0,0 1 0,-1 2 0,0-1 0,0-1 0,0 1 0,0-1 0,-1 1 0,1-1 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,1-1 0,-1 1 0,0-1 0,0 1 0,0-1 0,0 0 0,0 0 0,0-1 0,0 1 0,-1 0 0,1-1 0,0 0 0,-8 2 0,-16 0 15,-1-1 0,1-1 0,-44-4 0,-1 0-1440,59 3-5401</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="636.06">101 102 24575,'16'-1'0,"0"-1"0,-1-1 0,1-1 0,0 0 0,28-12 0,-25 9 0,0 0 0,1 2 0,24-5 0,77-2 15,88-14-1395,-186 22-5446</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">62 102 24575,'-3'2'0,"1"0"0,-1 0 0,0 0 0,1 1 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,-1 5 0,2-6 0,-2 4 0,-1 2 0,-1 1 0,2-1 0,-1 1 0,1 0 0,-3 16 0,5-23 0,1-1 0,0 1 0,0 0 0,0-1 0,0 1 0,0-1 0,0 1 0,0 0 0,1-1 0,-1 1 0,0-1 0,1 1 0,-1-1 0,1 1 0,-1-1 0,1 1 0,-1-1 0,1 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 1 0,0-2 0,1 1 0,-1 0 0,0 0 0,0 0 0,0-1 0,1 1 0,-1-1 0,1 1 0,-2-1 0,2 1 0,0-1 0,-1 0 0,0 0 0,2 0 0,20 3 0,-1-2 0,0 0 0,26-4 0,-27 1 0,0 1 0,1 1 0,33 5 0,-52-5 0,-1 1 0,0-1 0,0 0 0,1 1 0,-2 0 0,1-1 0,1 1 0,-2 0 0,1 0 0,1 0 0,-2 1 0,1-1 0,0 0 0,0 1 0,-1-1 0,0 1 0,1 0 0,0 0 0,-1 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,-1 1 0,1-1 0,0 0 0,-1 1 0,1-1 0,-1 1 0,1-1 0,-1 0 0,0 1 0,0-1 0,0 1 0,-1 2 0,0-1 0,0-1 0,0 1 0,1-1 0,-2 1 0,1-1 0,-1 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0-1 0,-1 1 0,1-1 0,-1 1 0,0-1 0,1 0 0,-1 0 0,1-1 0,-1 1 0,0 0 0,0-1 0,0 0 0,-6 2 0,-15 0 15,0-1 0,0-1 0,-37-4 0,-2 0-1440,52 3-5401</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="636.05">88 102 24575,'14'-1'0,"0"-1"0,-1-1 0,1-1 0,0 0 0,24-12 0,-21 9 0,-1 0 0,2 2 0,20-5 0,67-2 15,77-14-1395,-162 22-5446</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -2316,7 +2313,7 @@
       <inkml:brushProperty name="height" value="0.025" units="cm"/>
     </inkml:brush>
   </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">209 28 24575,'-4'-1'0,"-1"1"0,1-2 0,-1 1 0,1 0 0,0-1 0,0 0 0,-5-2 0,-25-10 0,30 14 0,-1 0 0,1-1 0,0 1 0,-1 1 0,1-1 0,0 1 0,-1-1 0,1 1 0,0 1 0,0-1 0,0 0 0,0 1 0,0 0 0,0 0 0,0 0 0,1 1 0,-1-1 0,1 1 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 0 0,1 1 0,-1-1 0,1 1 0,0 0 0,0 0 0,0 0 0,-2 8 0,-2 2 0,1 1 0,1-1 0,1 1 0,0 0 0,1 0 0,0 0 0,2 29 0,0-40 0,0 0 0,1-1 0,-1 1 0,1-1 0,0 1 0,1 0 0,-1-1 0,0 0 0,1 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,1-1 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,1-1 0,-1 1 0,0-1 0,1 0 0,-1 1 0,1-2 0,0 1 0,-1 0 0,1-1 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,-1-1 0,1 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,0-1 0,6-2 0,-8 3 0,0 1 0,0-1 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,0-1 0,0 1 0,0 0 0,0-2 0,0 2 0,-1-1 0,0 1 0,1-1 0,-1 1 0,0-1 0,0 1 0,0 0 0,-1-1 0,1 1 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,-1 0 0,-4-3 0,0 1 0,0 0 0,0 0 0,-1 1 0,1 0 0,-1 0 0,-7 0 0,11 2-114,1 0 1,0 0-1,0 0 0,-1 1 0,1-1 1,0 1-1,0 0 0,0 0 0,-1 0 1,1 0-1,-3 2 0,-4 4-6712</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">122 28 24575,'-2'-1'0,"-1"1"0,1-2 0,-1 1 0,1 0 0,-1-1 0,1 0 0,-3-2 0,-15-10 0,17 14 0,1 0 0,-1-1 0,1 1 0,-1 1 0,1-1 0,-1 1 0,0-1 0,1 1 0,0 1 0,-1-1 0,1 0 0,0 1 0,-1 0 0,1 0 0,0 0 0,0 1 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 1 0,1-1 0,-1 1 0,1 0 0,0 0 0,0 0 0,-1 8 0,-2 2 0,1 1 0,1-1 0,0 1 0,0 0 0,1 0 0,0 0 0,1 29 0,0-40 0,0 0 0,1-1 0,-1 1 0,0-1 0,1 1 0,0 0 0,0-1 0,-1 0 0,1 1 0,0-1 0,1 0 0,-1 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,1-1 0,0 1 0,-1-1 0,1 0 0,0 0 0,0 0 0,-1 0 0,2-1 0,-2 1 0,1-1 0,0 0 0,0 1 0,1-2 0,-1 1 0,0 0 0,0-1 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0-1 0,0 0 0,0 0 0,0 0 0,1 0 0,-2 0 0,1-1 0,3-2 0,-4 3 0,-1 1 0,1-1 0,0 1 0,-1-1 0,1 0 0,-1 1 0,1-1 0,0 0 0,-1 0 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0-2 0,0 2 0,0-1 0,-1 1 0,1-1 0,-1 1 0,1-1 0,-1 1 0,1 0 0,-1-1 0,0 1 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,-4-3 0,1 1 0,0 0 0,0 0 0,0 1 0,-1 0 0,1 0 0,-5 0 0,7 2-114,0 0 1,0 0-1,0 0 0,0 1 0,0-1 1,1 1-1,-1 0 0,0 0 0,0 0 1,0 0-1,-1 2 0,-3 4-6712</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -2343,7 +2340,7 @@
       <inkml:brushProperty name="height" value="0.025" units="cm"/>
     </inkml:brush>
   </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">1 121 24575,'39'-46'0,"-29"34"0,0 0 0,0 0 0,1 1 0,18-14 0,-29 25 0,1 0 0,-1 0 0,0-1 0,1 1 0,-1 0 0,0-1 0,1 1 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1-1 0,0 1 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,1 1 0,-1-1 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 1 0,1-1 0,-1 0 0,0 1 0,1-1 0,-1 0 0,0 0 0,1 1 0,5 21 0,-8 24 0,-24 112-1365,23-148-5461</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1 121 24575,'15'-46'0,"-11"34"0,-1 0 0,1 0 0,0 1 0,7-14 0,-11 25 0,1 0 0,-1 0 0,0-1 0,0 1 0,0 0 0,0-1 0,0 1 0,0 0 0,1 0 0,-1 0 0,0 0 0,0-1 0,0 1 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 1 0,1-1 0,-1 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 1 0,3 21 0,-4 24 0,-9 112-1365,9-148-5461</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -2370,8 +2367,8 @@
       <inkml:brushProperty name="height" value="0.025" units="cm"/>
     </inkml:brush>
   </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">1 46 24575,'5'-3'0,"1"-1"0,0 1 0,0 1 0,0-1 0,0 1 0,0 0 0,0 0 0,1 1 0,9-2 0,-1 0 0,11-3 0,0 2 0,0 0 0,0 2 0,40 1 0,-64 1 0,-1 0 0,1 0 0,-1 0 0,0 0 0,1 1 0,-1-1 0,0 1 0,0-1 0,1 1 0,-1 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,-1 0 0,1 0 0,0 0 0,0 3 0,0 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,0 1 0,0-1 0,0 0 0,-1 8 0,-2 1 0,0 1 0,-1 0 0,0-1 0,-8 18 0,-6 2-18,11-19-319,-1-1 0,2 1 1,-5 16-1,7-16-6489</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1224.68">75 165 24575,'13'-1'0,"1"0"0,-1-2 0,25-6 0,13-3 0,24-2-5,-44 7-449,0 2 1,54-3 0,-69 8-6373</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1 51 24575,'4'-4'0,"1"0"0,0 1 0,-1 0 0,1 0 0,0 1 0,0 0 0,0-1 0,0 2 0,8-2 0,-1 0 0,9-4 0,0 3 0,0-1 0,0 3 0,32 1 0,-52 1 0,0 0 0,1 0 0,-1 0 0,-1 0 0,2 1 0,-1-1 0,0 1 0,-1-1 0,2 1 0,-1 0 0,0-1 0,-1 2 0,1-1 0,0 0 0,0-1 0,0 1 0,-1 0 0,1 0 0,0 0 0,0 1 0,0-1 0,-1 1 0,0-1 0,1 0 0,0 3 0,0 1 0,0-1 0,0 0 0,-1 1 0,0-1 0,0 2 0,0-2 0,0 1 0,0 8 0,-3 1 0,1 2 0,-2-1 0,1-1 0,-6 21 0,-6 1-18,10-20-319,-2-2 0,2 1 1,-4 18-1,6-17-6489</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1224.67">60 182 24575,'11'-1'0,"0"0"0,0-3 0,19-5 0,11-5 0,19-1-5,-35 7-449,0 3 1,43-4 0,-55 9-6373</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -2453,7 +2450,7 @@
       <inkml:brushProperty name="height" value="0.025" units="cm"/>
     </inkml:brush>
   </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">0 58 24575,'0'1'0,"1"0"0,-1 0 0,1-1 0,-1 1 0,1 0 0,-1 0 0,1 0 0,-1-1 0,1 1 0,0 0 0,-1-1 0,1 1 0,0-1 0,0 1 0,-1-1 0,1 1 0,0-1 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,1 1 0,35-9 0,-29 4 0,1 0 0,-1 0 0,-1-1 0,1 0 0,-1-1 0,0 1 0,6-10 0,-9 12 0,-4 4 0,1 0 0,-1 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,4 19 0,-3 20 0,-4-5-248,-13 59-1,12-73-619,0 0-5958</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">0 58 24575,'0'1'0,"0"0"0,0 0 0,1-1 0,-1 1 0,0 0 0,0 0 0,1 0 0,-1-1 0,0 1 0,1 0 0,-1-1 0,0 1 0,0-1 0,1 1 0,-1-1 0,0 1 0,1-1 0,-1 1 0,0-1 0,1 0 0,-1 1 0,1-1 0,-1 0 0,0 0 0,1 0 0,-1 0 0,0 1 0,1-1 0,-1-1 0,1 1 0,-1 0 0,0 0 0,1 0 0,-1 0 0,1-1 0,0 1 0,14-9 0,-12 4 0,1 0 0,-1 0 0,0-1 0,1 0 0,-1-1 0,-1 1 0,4-10 0,-4 12 0,-2 4 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,2 19 0,-1 20 0,-3-5-248,-4 60-1,4-74-619,0 0-5958</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -2480,7 +2477,7 @@
       <inkml:brushProperty name="height" value="0.025" units="cm"/>
     </inkml:brush>
   </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">44 5 24575,'-1'7'0,"0"0"0,-1 0 0,1-1 0,-2 1 0,1 0 0,-1-1 0,-5 10 0,-8 22 0,15-35 0,0-1 0,0 1 0,0-1 0,0 1 0,1-1 0,-1 1 0,1 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0-1 0,1 1 0,-1 0 0,1-1 0,0 1 0,0-1 0,-1 1 0,2-1 0,-1 1 0,3 4 0,-1-5 0,0 0 0,0 0 0,0 0 0,1 0 0,-1-1 0,1 1 0,-1-1 0,1 0 0,0 0 0,-1 0 0,1-1 0,0 1 0,0-1 0,-1 0 0,6 0 0,-2 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0-1 0,0 0 0,0-1 0,0 1 0,0-1 0,-1 0 0,1-1 0,-1 0 0,0 0 0,0 0 0,0-1 0,0 0 0,0 0 0,-1 0 0,1-1 0,-1 0 0,0 0 0,-1 0 0,1 0 0,-1-1 0,0 0 0,-1 0 0,1 0 0,-1 0 0,4-12 0,-5 14 0,-1 0 0,1-1 0,-1 1 0,0 0 0,0 0 0,0 0 0,-1-1 0,1 1 0,-1 0 0,-1-6 0,1 8 0,-1 1 0,0-1 0,0 1 0,1 0 0,-1-1 0,0 1 0,0 0 0,-1-1 0,1 1 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 1 0,-1-1 0,1 0 0,-1 1 0,1-1 0,-1 1 0,0-1 0,1 1 0,-1 0 0,1 0 0,-1 0 0,0 0 0,1 0 0,-4 0 0,-91 3-1365,83-3-5461</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">29 5 24575,'0'7'0,"-1"0"0,0 0 0,0-1 0,-1 1 0,1 0 0,-1-1 0,-4 10 0,-4 22 0,9-35 0,1-1 0,-1 1 0,0-1 0,1 1 0,0-1 0,-1 1 0,1 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0-1 0,1 1 0,-1 0 0,0-1 0,1 1 0,0-1 0,-1 1 0,1-1 0,0 1 0,1 4 0,0-5 0,0 0 0,0 0 0,0 0 0,1 0 0,-1-1 0,0 1 0,0-1 0,1 0 0,0 0 0,-1 0 0,0-1 0,1 1 0,-1-1 0,0 0 0,4 0 0,-1 1 0,0-1 0,-1 0 0,1 0 0,-1 0 0,1-1 0,0 0 0,-1-1 0,1 1 0,-1-1 0,0 0 0,1-1 0,-1 0 0,0 0 0,0 0 0,0-1 0,0 0 0,0 0 0,-1 0 0,1-1 0,-1 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 0 0,-1 0 0,0 0 0,0 0 0,3-12 0,-4 14 0,0 0 0,0-1 0,0 1 0,-1 0 0,1 0 0,0 0 0,-1-1 0,0 1 0,0 0 0,0-6 0,0 8 0,-1 1 0,0-1 0,1 1 0,0 0 0,-1-1 0,0 1 0,1 0 0,-2-1 0,2 1 0,-1 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,0 1 0,-1-1 0,2 1 0,-2 0 0,2 0 0,-2 0 0,1 0 0,0 0 0,-2 0 0,-60 3-1365,54-3-5461</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -2507,8 +2504,8 @@
       <inkml:brushProperty name="height" value="0.025" units="cm"/>
     </inkml:brush>
   </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">1 257 24575,'6'-2'0,"1"-1"0,-1 0 0,0 0 0,0 0 0,-1-1 0,1 0 0,-1 0 0,0 0 0,0-1 0,8-9 0,-10 12 0,32-48 0,-17 23 0,-24 91 0,-45 145-1365,46-191-5461</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="842.79">417 228 24575,'1'-4'0,"1"0"0,-1 0 0,1 0 0,0 0 0,0 1 0,0-1 0,0 1 0,0 0 0,1-1 0,6-5 0,-1 0 0,108-159 0,-116 168 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,2 16 0,-6 19 0,-25 53 26,21-67-304,0 0 0,1 1-1,2 0 1,-6 42 0,10-52-6548</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1 274 24575,'5'-2'0,"1"-1"0,-1 0 0,0-1 0,0 1 0,0-1 0,0 0 0,-1-1 0,0 1 0,0-1 0,7-10 0,-8 13 0,27-52 0,-15 26 0,-20 96 0,-38 155-1365,38-204-5461</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="842.79">354 243 24575,'1'-4'0,"1"0"0,-1-1 0,0 1 0,1 0 0,0 1 0,-1-2 0,1 2 0,0 0 0,0-1 0,6-6 0,-1 0 0,91-169 0,-98 179 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,2 17 0,-5 20 0,-22 57 26,18-71-304,1-1 0,0 2-1,1-1 1,-4 45 0,8-55-6548</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -2535,7 +2532,7 @@
       <inkml:brushProperty name="height" value="0.025" units="cm"/>
     </inkml:brush>
   </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">0 21 24575,'1'0'0,"0"1"0,-1-1 0,1 0 0,0 1 0,-1-1 0,1 1 0,0-1 0,-1 1 0,1-1 0,-1 1 0,1-1 0,-1 1 0,1-1 0,-1 1 0,1 0 0,-1-1 0,0 1 0,1 0 0,-1 0 0,0-1 0,1 1 0,-1 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 1 0,3 25 0,-3-22 0,1-10 0,0 2 0,0 0 0,0 0 0,0 1 0,1-1 0,-1 0 0,1 0 0,0 1 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,1 0 0,4-3 0,-4 4 0,-1 0 0,0-1 0,0 1 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 1 0,1-1 0,0 1 0,-1-1 0,1 1 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 1 0,-1-1 0,1 1 0,2 0 0,-5-1 0,1 0 0,-1 1 0,0-1 0,1 0 0,-1 0 0,0 0 0,0 1 0,1-1 0,-1 0 0,0 0 0,0 1 0,1-1 0,-1 0 0,0 0 0,0 1 0,0-1 0,0 0 0,1 1 0,-1-1 0,0 0 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,0 0 0,0 1 0,-1-1 0,1 0 0,0 1 0,-15 13 0,-21 3 0,35-17 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1-1 0,0 1 0,1 0 0,-1 0 0,0-1 0,1 1 0,-1 0 0,0-1 0,1 1 0,-1-1 0,1 1 0,-1-1 0,1 1 0,-1-1 0,1 1 0,0-1 0,-1 1 0,1-1 0,-1 0 0,1 1 0,0-1 0,0 0 0,-1 1 0,1-1 0,0 0 0,0 1 0,0-1 0,0-1 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,1 0 0,-1-1 0,1 1 0,0 0 0,-1 0 0,3-4 0,-2 5 0,-1 0 0,0 1 0,0-1 0,1 0 0,-1 1 0,1-1 0,-1 0 0,0 1 0,1-1 0,-1 1 0,1-1 0,0 1 0,-1-1 0,1 1 0,-1-1 0,1 1 0,0-1 0,-1 1 0,1 0 0,0-1 0,-1 1 0,1 0 0,0 0 0,0-1 0,1 1 0,-1 1 0,0 0 0,0 0 0,-1 0 0,1 1 0,0-1 0,0 0 0,-1 0 0,1 1 0,0-1 0,-1 0 0,1 0 0,-1 1 0,0-1 0,0 1 0,1-1 0,-1 0 0,0 1 0,0-1 0,0 1 0,0-1 0,0 0 0,-1 2 0,1-2-45,0 1-1,0-1 1,1 0-1,-1 0 1,-1 0-1,1 1 1,0-1-1,0 0 1,0 0-1,-1 0 1,1 1-1,0-1 1,-1 0-1,1 0 1,-1 0-1,1 0 1,-1 0-1,0 0 1,1 0-1,-1 0 1,0 0-1,0 0 1,0 0-1,0-1 0,0 1 1,0 0-1,0-1 1,0 1-1,-1 0 1,-3-2-6781</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">0 29 24575,'1'0'0,"0"2"0,-1-2 0,1 0 0,0 1 0,-1-1 0,1 1 0,0-1 0,-1 2 0,1-2 0,-1 1 0,1-1 0,-1 2 0,1-2 0,-1 1 0,1 0 0,-1-1 0,0 2 0,1-1 0,-1 0 0,0-1 0,1 2 0,-1-1 0,0 1 0,0-2 0,0 1 0,0 0 0,0 2 0,3 35 0,-3-31 0,1-14 0,0 3 0,0-1 0,0 1 0,0 1 0,1-1 0,-1 0 0,1 0 0,0 1 0,0-1 0,0 1 0,0 0 0,0 1 0,0-1 0,1 0 0,-1 0 0,1 1 0,4-5 0,-4 5 0,-1 1 0,0-2 0,0 2 0,1-1 0,-1 1 0,0-1 0,1 1 0,-1 1 0,1-1 0,0 1 0,-1-2 0,1 2 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 2 0,-1-2 0,1 1 0,2 0 0,-5-1 0,1 0 0,-1 2 0,0-2 0,1 0 0,-1 0 0,0 0 0,0 1 0,1-1 0,-1 0 0,0 0 0,0 2 0,1-2 0,-1 0 0,0 0 0,0 1 0,0-1 0,0 0 0,1 1 0,-1-1 0,0 0 0,0 2 0,0-2 0,0 0 0,0 1 0,0-1 0,0 0 0,0 2 0,0-2 0,0 0 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,0 0 0,0 2 0,-1-2 0,1 0 0,0 1 0,-15 19 0,-21 3 0,35-23 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1-1 0,0 1 0,1 0 0,-1 0 0,0-2 0,1 2 0,-1 0 0,0-1 0,1 1 0,-1-1 0,1 1 0,-1-2 0,1 2 0,-1-1 0,1 1 0,0-2 0,-1 2 0,1-1 0,-1 0 0,1 1 0,0-2 0,0 1 0,-1 1 0,1-2 0,0 1 0,0 1 0,0-1 0,0-2 0,0 0 0,0 0 0,0-1 0,0 1 0,0 1 0,1-1 0,-1-1 0,1 1 0,0 0 0,-1 0 0,3-5 0,-2 7 0,-1-1 0,0 2 0,0-1 0,1 0 0,-1 1 0,1-2 0,-1 1 0,0 1 0,1-2 0,-1 2 0,1-1 0,0 1 0,-1-1 0,1 1 0,-1-2 0,1 2 0,0-1 0,-1 1 0,1 0 0,0-2 0,-1 2 0,1 0 0,0 0 0,0-1 0,1 1 0,-1 1 0,0 1 0,0-1 0,-1 1 0,1 0 0,0 0 0,0-1 0,-1 1 0,1 0 0,0 0 0,-1-1 0,1 0 0,-1 2 0,0-1 0,0 0 0,1 0 0,-1-1 0,0 2 0,0-2 0,0 2 0,0-1 0,0-1 0,-1 3 0,1-3-45,0 2-1,0-1 1,1-1-1,-1 0 1,-1 1-1,1 1 1,0-2-1,0 0 1,0 1-1,-1-1 1,1 2-1,0-2 1,-1 1-1,1-1 1,-1 0-1,1 1 1,-1-1-1,0 1 1,1-1-1,-1 0 1,0 1-1,0-1 1,0 1-1,0-2 0,0 1 1,0 0-1,0-1 1,0 2-1,-1-1 1,-3-2-6781</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -2562,13 +2559,13 @@
       <inkml:brushProperty name="height" value="0.025" units="cm"/>
     </inkml:brush>
   </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">120 0 24575,'-2'8'0,"0"-1"0,-1 1 0,1-1 0,-1 0 0,-1 1 0,1-2 0,-1 1 0,-1 0 0,-6 8 0,-4 7 0,5-4 0,1 1 0,0 0 0,2 0 0,0 1 0,1 0 0,1 0 0,1 0 0,0 1 0,2-1 0,0 39 0,3-56 3,-1 1 0,1 0 0,1 0 0,-1-1 0,1 1 0,-1 0 0,1-1 0,0 1-1,0-1 1,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,0-1 0,4 3 0,65 38-308,-42-27-808,-20-10-5713</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1028.44">340 178 24575,'0'11'0,"-2"1"0,0-1 0,0 0 0,-6 16 0,-5 32 0,11-44 0,1 0 0,1 1 0,1-1 0,0 1 0,4 18 0,-4-31 0,-1-1 0,1 1 0,0-1 0,0 1 0,0-1 0,0 0 0,0 0 0,0 1 0,0-1 0,1 0 0,0 0 0,-1 0 0,1 0 0,0-1 0,0 1 0,3 3 0,-2-5 0,-1 1 0,0-1 0,1 1 0,-1-1 0,0 0 0,1 0 0,-1 1 0,0-2 0,1 1 0,-1 0 0,0 0 0,1-1 0,-1 0 0,0 1 0,0-1 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0-1 0,2-1 0,1 0 0,0-1 0,0 0 0,-1 0 0,1-1 0,-1 0 0,0 1 0,0-1 0,-1 0 0,0-1 0,1 1 0,-2-1 0,1 1 0,-1-1 0,1 0 0,-2 0 0,1 0 0,-1 0 0,1-7 0,1-11 0,-2 0 0,-1 0 0,-3-32 0,2 42 0,1 12-57,0 0 0,0 0 1,0 0-1,0 1 0,-1-1 0,1 0 0,0 1 0,-1-1 0,1 0 0,-1 1 0,0-1 1,0 0-1,1 1 0,-1-1 0,0 1 0,0-1 0,-1 1 0,1 0 0,0-1 1,0 1-1,-1 0 0,1 0 0,-3-2 0,-8-1-6769</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1727.32">561 429 24575,'0'2'0,"0"4"0,3 3 0,0 3 0,0 1 0,0 2 0,-1 0 0,-1 1 0,-1-1 0,1 0 0,-4 0 0,0 1 0,-3-4 0,-3-3 0,1-1 0,-2 1 0,2-1-8191</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="2649.35">826 281 24575,'-14'126'0,"7"-67"0,4-42 0,1 0 0,0 0 0,1 0 0,1 0 0,3 23 0,-3-38 0,0 0 0,1 0 0,-1-1 0,1 1 0,-1 0 0,1 0 0,0-1 0,0 1 0,-1-1 0,1 1 0,0 0 0,1-1 0,-1 0 0,0 1 0,0-1 0,1 0 0,-1 1 0,1-1 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1-1 0,1 1 0,0 0 0,0-1 0,-1 1 0,1-1 0,0 1 0,0-1 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,0-1 0,-1 1 0,1-1 0,3 0 0,0 0 0,0-1 0,0 0 0,0 0 0,0 0 0,0-1 0,-1 0 0,1 0 0,-1 0 0,0 0 0,0-1 0,0 1 0,7-9 0,-5 1 0,0 0 0,-1-1 0,0 1 0,-1-1 0,-1 0 0,1 0 0,-2-1 0,0 1 0,0-1 0,-1 1 0,-1-1 0,0 1 0,-1-1 0,0 1 0,-4-20 0,3 28-85,0 0 0,0-1-1,0 1 1,-1 0 0,1 0-1,-1 0 1,0 0 0,0 1-1,0-1 1,-1 1 0,1 0-1,-1 0 1,0 0 0,0 0-1,-8-4 1,4 2-6741</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="3220.54">1121 592 24575,'0'5'0,"0"4"0,0 3 0,0 2 0,0 4 0,0 1 0,0 0 0,-3-3 0,0-2 0,0-1 0,-3-3 0,1 0 0,1-2-8191</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="4032.63">1282 399 24575,'-15'162'0,"15"-152"0,1 0 0,0 0 0,0 0 0,5 18 0,-6-27 0,0 0 0,0 0 0,1 1 0,-1-1 0,0 0 0,1 0 0,-1 0 0,0 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,0-1 0,0 1 0,0 0 0,-1-1 0,1 1 0,0 0 0,0-1 0,1 1 0,-1-1 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,1 1 0,-1 0 0,0-1 0,0 1 0,0-1 0,0 1 0,0-1 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,-1 0 0,1 0 0,1-2 0,1 0 0,0 0 0,0-1 0,0 1 0,-1-1 0,0 0 0,1 0 0,-2 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,0-6 0,7-59 0,-7 50 0,1-6-117,4-45 364,-6 64-396,-1 1-1,0-1 1,-1 1-1,1-1 1,-1 1-1,0 0 1,-1-1-1,1 1 0,-5-9 1,0 4-6677</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="4765.13">1547 237 24575,'3'36'0,"1"0"0,2-1 0,15 54 0,0 2 0,-14-51 0,-1 0 0,-1 0 0,-3 0 0,-3 61 0,0-96 7,0 0-1,-1 0 0,1 0 0,-1-1 1,0 1-1,-1 0 0,1-1 1,-1 1-1,1-1 0,-1 0 1,-1 0-1,1 0 0,-1 0 0,1-1 1,-1 0-1,0 1 0,0-1 1,-6 3-1,-5 3-303,0 0 0,-1-1 0,0-1 0,-18 5 0,25-9-6529</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">102 0 24575,'-2'9'0,"0"-2"0,0 2 0,0-2 0,0 0 0,-2 2 0,2-3 0,-2 2 0,0-1 0,-5 9 0,-4 8 0,5-5 0,0 1 0,0 0 0,2 1 0,0 0 0,1 0 0,1 1 0,1-1 0,-1 1 0,3 0 0,-1 40 0,3-58 3,-1 0 0,1 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0-1 0,1 2-1,0-2 1,0 0 0,0 0 0,1 0 0,-2 1 0,2-1 0,-1 0 0,1-1 0,3 3 0,55 41-308,-36-29-808,-16-10-5713</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1028.44">288 190 24575,'0'11'0,"-2"2"0,1-1 0,-1 0 0,-5 16 0,-4 35 0,10-47 0,0 0 0,1 1 0,1-1 0,-1 1 0,5 20 0,-4-34 0,-1-1 0,0 1 0,1-1 0,0 1 0,0-1 0,0 1 0,0-1 0,-1 1 0,1-1 0,1 0 0,0 0 0,-1 0 0,0 1 0,1-2 0,0 1 0,2 3 0,-2-5 0,0 1 0,0-1 0,0 1 0,0-1 0,0 0 0,0 0 0,0 1 0,0-2 0,0 1 0,0 0 0,0 0 0,0-1 0,0 0 0,0 1 0,-1-1 0,2 0 0,-2 0 0,1 0 0,0 0 0,0 0 0,-1-1 0,3-2 0,0 1 0,0-1 0,0 0 0,0-1 0,0 0 0,-1 0 0,1 1 0,-1-2 0,0 1 0,-1-2 0,2 2 0,-3-1 0,2 0 0,-1 0 0,0 0 0,-1-1 0,1 1 0,-2-1 0,2-6 0,1-13 0,-2 0 0,-1 1 0,-3-35 0,2 45 0,1 13-57,0 0 0,0 0 1,0 0-1,0 1 0,-1-1 0,1-1 0,0 2 0,-1-1 0,1 0 0,0 1 0,-1-1 1,0 0-1,1 1 0,-1-1 0,0 1 0,0-2 0,0 2 0,0 0 0,0-1 1,0 1-1,-1 0 0,2 0 0,-4-2 0,-6-2-6769</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1727.32">475 457 24575,'0'2'0,"0"5"0,3 2 0,-1 4 0,1 1 0,0 2 0,-2 0 0,0 1 0,-1-1 0,1 0 0,-4 0 0,1 1 0,-3-4 0,-3-4 0,1 0 0,-1 0 0,1 0-8191</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="2649.35">700 299 24575,'-12'135'0,"6"-72"0,4-45 0,0 0 0,0 0 0,1 0 0,1 0 0,3 25 0,-3-41 0,0 0 0,1 0 0,-1-1 0,1 1 0,-1 0 0,0 1 0,1-2 0,0 1 0,-1-1 0,1 1 0,0 0 0,0-1 0,0 0 0,0 1 0,0-1 0,1 0 0,-1 2 0,0-2 0,0 0 0,1 0 0,-1 0 0,0 0 0,0-1 0,1 1 0,0 0 0,-1-1 0,0 1 0,1-1 0,-1 1 0,1-1 0,0 0 0,0 0 0,-2 0 0,2 0 0,0 0 0,-1 0 0,1-1 0,-1 1 0,1-1 0,2 0 0,0 0 0,0-1 0,1 0 0,-1 0 0,0-1 0,0 0 0,0 0 0,0 0 0,-1 0 0,1-1 0,-1 0 0,1 1 0,5-10 0,-4 1 0,0 1 0,-1-2 0,1 1 0,-2-1 0,-1 1 0,2-1 0,-2-1 0,-1 1 0,1-1 0,-1 2 0,-1-2 0,0 1 0,-1-1 0,0 1 0,-3-21 0,2 30-85,0 0 0,1-2-1,-1 2 1,0 0 0,0 0-1,-1-1 1,1 1 0,-1 1-1,1-1 1,-2 0 0,2 1-1,-2 0 1,1 0 0,0 0-1,-8-5 1,5 3-6741</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="3220.54">950 631 24575,'0'5'0,"0"5"0,0 2 0,0 3 0,0 5 0,0 0 0,0 0 0,-3-3 0,1-2 0,-1-1 0,-2-3 0,1-1 0,0-1-8191</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="4032.63">1086 425 24575,'-13'173'0,"13"-163"0,1 1 0,0 0 0,0-1 0,4 20 0,-5-29 0,0 0 0,0 0 0,1 2 0,-1-2 0,0 0 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,0-1 0,0 1 0,-1 1 0,0-2 0,1 1 0,0 0 0,0-1 0,1 1 0,-2-1 0,1 1 0,0-1 0,0 0 0,0 1 0,0-1 0,0 0 0,-1 0 0,2 0 0,-1 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,0-1 0,1 1 0,-1 0 0,0-1 0,-1 1 0,1-1 0,0 1 0,0-1 0,0 1 0,0-1 0,-1-1 0,1 2 0,0-1 0,-1 0 0,1 0 0,1-2 0,0 0 0,1 0 0,-1-2 0,1 2 0,-1-1 0,-1 0 0,2-1 0,-2 1 0,0 0 0,1 0 0,-1-1 0,1 1 0,-1-7 0,7-62 0,-6 53 0,0-7-117,4-48 364,-5 69-396,-1 1-1,0-2 1,-1 2-1,1-1 1,-1 0-1,0 1 1,0-1-1,0 0 0,-4-9 1,0 5-6677</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="4765.13">1311 253 24575,'2'38'0,"2"0"0,1 0 0,12 56 0,1 3 0,-12-54 0,-1 0 0,-1-1 0,-2 1 0,-3 64 0,0-101 7,1-1-1,-2 0 0,1 1 0,-1-2 1,1 1-1,-2 1 0,1-2 1,0 1-1,0-1 0,0 1 1,-2-1-1,2 0 0,-2 1 0,2-2 1,-2 0-1,1 1 0,0-1 1,-6 4-1,-4 2-303,1 1 0,-2-2 0,1 0 0,-16 5 0,21-10-6529</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -2732,8 +2729,8 @@
       <inkml:brushProperty name="height" value="0.025" units="cm"/>
     </inkml:brush>
   </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">1 2 24575,'55'-1'0,"59"2"0,-112-1 0,-1 0 0,1 0 0,0 1 0,-1-1 0,1 0 0,-1 1 0,1-1 0,-1 1 0,1 0 0,-1-1 0,1 1 0,-1 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 1 0,-1-1 0,1 0 0,1 2 0,-1 0 0,0 0 0,-1 0 0,1 1 0,-1-1 0,1 0 0,-1 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,-2 5 0,-2 7 0,0-1 0,-1-1 0,-14 27 0,-23 47 0,38-77-1365,0-1-5461</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="983.57">25 170 24575,'2'0'0,"3"0"0,2 0 0,3 0 0,0 0 0,2 0 0,1 2 0,-1 1 0,-1 2 0,-2-1 0,1 3 0,-2 0 0,0 1 0,-1 0 0,-1-2 0,2-1 0,-1-1-8191</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1 2 24575,'33'-1'0,"36"2"0,-67-1 0,-2 0 0,1 0 0,1 1 0,-2-1 0,1 0 0,0 1 0,0-1 0,0 1 0,0 0 0,0-1 0,0 1 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,-1 1 0,0-1 0,1 0 0,0 2 0,0 0 0,-1 0 0,0 0 0,1 1 0,-1-1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,-1 5 0,-2 7 0,1-1 0,-1-1 0,-9 27 0,-13 47 0,22-77-1365,1-1-5461</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="983.57">16 170 24575,'1'0'0,"2"0"0,1 0 0,2 0 0,0 0 0,1 0 0,1 2 0,0 1 0,-2 2 0,0-1 0,0 3 0,-1 0 0,-1 1 0,1 0 0,-2-2 0,2-1 0,-1-1-8191</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -2760,7 +2757,7 @@
       <inkml:brushProperty name="height" value="0.025" units="cm"/>
     </inkml:brush>
   </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">140 46 24575,'-1'0'0,"-8"0"0,0 0 0,0 1 0,0 0 0,0 0 0,-9 3 0,15-3 0,1-1 0,0 1 0,-1 0 0,1 1 0,0-1 0,0 0 0,0 0 0,0 1 0,0 0 0,0-1 0,1 1 0,-1 0 0,0 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 5 0,1-4 0,1-1 0,0 1 0,0 0 0,0 0 0,0-1 0,0 1 0,1-1 0,-1 1 0,1-1 0,0 1 0,-1-1 0,1 0 0,0 0 0,1 0 0,-1 0 0,4 3 0,17 20 0,-3 9 0,12 22 0,-30-52 0,0-1 0,-1 1 0,1 0 0,-1-1 0,0 1 0,0 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-2 7 0,0-9 0,0 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0-1 0,0 0 0,0 0 0,-1 1 0,1-1 0,0 0 0,-1-1 0,1 1 0,0 0 0,-1-1 0,1 1 0,-1-1 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-4-1 0,1 1 0,1 0 0,0-1 0,0 1 0,0-1 0,0 1 0,0-1 0,0 0 0,1-1 0,-1 1 0,0-1 0,0 1 0,1-1 0,-1 0 0,1-1 0,0 1 0,-1 0 0,-4-6 0,6 5 0,1 0 0,-1 0 0,0-1 0,1 1 0,0-1 0,0 1 0,0-1 0,0 1 0,0-1 0,1 0 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,1 0 0,-1 1 0,1-1 0,0 1 0,0-1 0,1 1 0,-1-1 0,1 1 0,2-4 0,4-5 0,2 0 0,-1 1 0,1 0 0,23-18 0,-25 23 0,-1 0 0,0 0 0,0-1 0,0 1 0,-1-1 0,0-1 0,0 0 0,-1 1 0,0-2 0,0 1 0,5-14 0,-7-13-1365,-3 25-5461</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">74 46 24575,'-1'0'0,"-3"0"0,-1 0 0,0 1 0,0 0 0,1 0 0,-6 3 0,9-3 0,0-1 0,0 1 0,-1 0 0,1 1 0,0-1 0,0 0 0,0 0 0,0 1 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,1 0 0,-1 1 0,1-1 0,-1 5 0,1-4 0,1-1 0,-1 1 0,1 0 0,-1 0 0,1-1 0,-1 1 0,2-1 0,-2 1 0,1-1 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,3 3 0,8 20 0,-2 9 0,7 22 0,-16-52 0,0-1 0,-1 1 0,2 0 0,-2-1 0,1 1 0,-1 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 7 0,-1-9 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0-1 0,0 0 0,0 0 0,-1 1 0,1-1 0,0 0 0,0-1 0,0 1 0,0 0 0,-1-1 0,1 1 0,0-1 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,-2-1 0,0 1 0,1 0 0,0-1 0,0 1 0,0-1 0,0 1 0,0-1 0,0 0 0,0-1 0,0 1 0,0-1 0,0 1 0,0-1 0,0 0 0,1-1 0,-1 1 0,0 0 0,-2-6 0,3 5 0,0 0 0,0 0 0,0-1 0,1 1 0,-1-1 0,1 1 0,-1-1 0,1 1 0,-1-1 0,1 0 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,1 0 0,-1 1 0,0-1 0,1 1 0,-1-1 0,1 1 0,0-1 0,0 1 0,1-4 0,2-5 0,1 0 0,0 1 0,0 0 0,12-18 0,-12 23 0,-2 0 0,1 0 0,0-1 0,-1 1 0,1-1 0,-1-1 0,0 0 0,-1 1 0,1-2 0,0 1 0,2-14 0,-4-13-1365,-1 25-5461</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -3081,15 +3078,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{678D5E9C-FA82-4BF1-AC9A-DE1452D6BB4F}">
-  <dimension ref="J1:BX26"/>
-  <sheetFormatPr defaultColWidth="2.5" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <dimension ref="J1:BV26"/>
+  <sheetFormatPr defaultColWidth="2.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="36" max="36" width="2.875" bestFit="1" customWidth="1"/>
-    <col min="52" max="53" width="2.875" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="2.875" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="2.85546875" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="3.140625" bestFit="1" customWidth="1"/>
+    <col min="52" max="53" width="2.85546875" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="2.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="10:74" x14ac:dyDescent="0.2">
+    <row r="1" spans="10:74" x14ac:dyDescent="0.25">
       <c r="AK1" t="s">
         <v>5</v>
       </c>
@@ -3097,15 +3095,13 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="10:74" x14ac:dyDescent="0.2">
-      <c r="M2" s="5"/>
+    <row r="2" spans="10:74" x14ac:dyDescent="0.25">
       <c r="R2" t="s">
         <v>0</v>
       </c>
       <c r="S2" t="s">
         <v>1</v>
       </c>
-      <c r="AG2" s="5"/>
       <c r="AK2" t="s">
         <v>0</v>
       </c>
@@ -3125,11 +3121,11 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="10:74" x14ac:dyDescent="0.2">
-      <c r="J3" s="7"/>
+    <row r="3" spans="10:74" x14ac:dyDescent="0.25">
+      <c r="J3" s="6"/>
       <c r="K3" s="3"/>
       <c r="L3" s="3"/>
-      <c r="M3" s="6"/>
+      <c r="M3" s="5"/>
       <c r="Q3">
         <v>0</v>
       </c>
@@ -3139,14 +3135,14 @@
       <c r="S3">
         <v>4</v>
       </c>
-      <c r="Z3" s="9"/>
-      <c r="AA3" s="10"/>
-      <c r="AB3" s="10"/>
-      <c r="AC3" s="10"/>
-      <c r="AD3" s="10"/>
-      <c r="AE3" s="10"/>
-      <c r="AF3" s="10"/>
-      <c r="AG3" s="16"/>
+      <c r="Z3" s="7"/>
+      <c r="AA3" s="8"/>
+      <c r="AB3" s="8"/>
+      <c r="AC3" s="8"/>
+      <c r="AD3" s="8"/>
+      <c r="AE3" s="8"/>
+      <c r="AF3" s="8"/>
+      <c r="AG3" s="13"/>
       <c r="AJ3">
         <v>0</v>
       </c>
@@ -3172,16 +3168,16 @@
         <v>0</v>
       </c>
       <c r="BA3">
+        <v>2</v>
+      </c>
+      <c r="BB3">
         <v>1</v>
-      </c>
-      <c r="BB3">
-        <v>2</v>
       </c>
       <c r="BC3">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="10:74" x14ac:dyDescent="0.2">
+    <row r="4" spans="10:74" x14ac:dyDescent="0.25">
       <c r="J4" s="1"/>
       <c r="Q4">
         <v>1</v>
@@ -3192,14 +3188,13 @@
       <c r="S4">
         <v>4</v>
       </c>
-      <c r="Z4" s="14"/>
-      <c r="AA4" s="5"/>
-      <c r="AB4" s="12"/>
-      <c r="AC4" s="12"/>
-      <c r="AD4" s="12"/>
-      <c r="AE4" s="12"/>
-      <c r="AF4" s="12"/>
-      <c r="AG4" s="13"/>
+      <c r="Z4" s="4"/>
+      <c r="AB4" s="10"/>
+      <c r="AC4" s="10"/>
+      <c r="AD4" s="10"/>
+      <c r="AE4" s="10"/>
+      <c r="AF4" s="10"/>
+      <c r="AG4" s="11"/>
       <c r="AJ4">
         <v>1</v>
       </c>
@@ -3225,18 +3220,17 @@
         <v>1</v>
       </c>
       <c r="BA4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="BB4">
         <v>1</v>
       </c>
       <c r="BC4">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
-    <row r="5" spans="10:74" x14ac:dyDescent="0.2">
+    <row r="5" spans="10:74" x14ac:dyDescent="0.25">
       <c r="J5" s="1"/>
-      <c r="M5" s="5"/>
       <c r="Q5">
         <v>2</v>
       </c>
@@ -3246,8 +3240,8 @@
       <c r="S5">
         <v>3</v>
       </c>
-      <c r="Z5" s="14"/>
-      <c r="AA5" s="15"/>
+      <c r="Z5" s="4"/>
+      <c r="AA5" s="12"/>
       <c r="AJ5">
         <v>2</v>
       </c>
@@ -3273,20 +3267,20 @@
         <v>2</v>
       </c>
       <c r="BA5">
+        <v>1</v>
+      </c>
+      <c r="BB5">
         <v>0</v>
-      </c>
-      <c r="BB5">
-        <v>1</v>
       </c>
       <c r="BC5">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="10:74" x14ac:dyDescent="0.2">
+    <row r="6" spans="10:74" x14ac:dyDescent="0.25">
       <c r="J6" s="4"/>
       <c r="K6" s="3"/>
       <c r="L6" s="3"/>
-      <c r="M6" s="6"/>
+      <c r="M6" s="5"/>
       <c r="Q6">
         <v>3</v>
       </c>
@@ -3296,8 +3290,8 @@
       <c r="S6">
         <v>3</v>
       </c>
-      <c r="Z6" s="14"/>
-      <c r="AA6" s="15"/>
+      <c r="Z6" s="4"/>
+      <c r="AA6" s="12"/>
       <c r="AJ6">
         <v>3</v>
       </c>
@@ -3319,21 +3313,20 @@
       <c r="AV6">
         <v>1</v>
       </c>
-      <c r="AX6" s="5"/>
       <c r="AZ6">
         <v>3</v>
       </c>
       <c r="BA6">
+        <v>3</v>
+      </c>
+      <c r="BB6">
         <v>0</v>
-      </c>
-      <c r="BB6">
-        <v>3</v>
       </c>
       <c r="BC6">
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="10:74" x14ac:dyDescent="0.2">
+    <row r="7" spans="10:74" x14ac:dyDescent="0.25">
       <c r="J7" s="1"/>
       <c r="Q7">
         <v>4</v>
@@ -3344,8 +3337,8 @@
       <c r="S7">
         <v>1</v>
       </c>
-      <c r="Z7" s="14"/>
-      <c r="AA7" s="15"/>
+      <c r="Z7" s="4"/>
+      <c r="AA7" s="12"/>
       <c r="AJ7">
         <v>4</v>
       </c>
@@ -3371,16 +3364,16 @@
         <v>4</v>
       </c>
       <c r="BA7">
+        <v>8</v>
+      </c>
+      <c r="BB7">
         <v>0</v>
-      </c>
-      <c r="BB7">
-        <v>8</v>
       </c>
       <c r="BC7">
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="10:74" x14ac:dyDescent="0.2">
+    <row r="8" spans="10:74" x14ac:dyDescent="0.25">
       <c r="J8" s="1"/>
       <c r="Q8">
         <v>5</v>
@@ -3391,9 +3384,8 @@
       <c r="S8">
         <v>1</v>
       </c>
-      <c r="Z8" s="14"/>
-      <c r="AA8" s="15"/>
-      <c r="AG8" s="5"/>
+      <c r="Z8" s="4"/>
+      <c r="AA8" s="12"/>
       <c r="AJ8">
         <v>5</v>
       </c>
@@ -3419,16 +3411,16 @@
         <v>5</v>
       </c>
       <c r="BA8">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="BB8">
         <v>5</v>
       </c>
       <c r="BC8">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
-    <row r="9" spans="10:74" x14ac:dyDescent="0.2">
+    <row r="9" spans="10:74" x14ac:dyDescent="0.25">
       <c r="J9" s="1"/>
       <c r="Q9">
         <v>6</v>
@@ -3439,14 +3431,13 @@
       <c r="S9">
         <v>-1</v>
       </c>
-      <c r="Z9" s="14"/>
-      <c r="AA9" s="5"/>
-      <c r="AB9" s="10"/>
-      <c r="AC9" s="10"/>
-      <c r="AD9" s="10"/>
-      <c r="AE9" s="10"/>
-      <c r="AF9" s="10"/>
-      <c r="AG9" s="16"/>
+      <c r="Z9" s="4"/>
+      <c r="AB9" s="8"/>
+      <c r="AC9" s="8"/>
+      <c r="AD9" s="8"/>
+      <c r="AE9" s="8"/>
+      <c r="AF9" s="8"/>
+      <c r="AG9" s="13"/>
       <c r="AJ9">
         <v>6</v>
       </c>
@@ -3472,24 +3463,24 @@
         <v>6</v>
       </c>
       <c r="BA9">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="BB9">
         <v>6</v>
       </c>
       <c r="BC9">
-        <v>9</v>
-      </c>
-      <c r="BO9" s="9"/>
-      <c r="BP9" s="10"/>
-      <c r="BQ9" s="10"/>
-      <c r="BR9" s="10"/>
-      <c r="BS9" s="10"/>
-      <c r="BT9" s="10"/>
-      <c r="BU9" s="10"/>
-      <c r="BV9" s="16"/>
+        <v>8</v>
+      </c>
+      <c r="BO9" s="7"/>
+      <c r="BP9" s="8"/>
+      <c r="BQ9" s="8"/>
+      <c r="BR9" s="8"/>
+      <c r="BS9" s="8"/>
+      <c r="BT9" s="8"/>
+      <c r="BU9" s="8"/>
+      <c r="BV9" s="13"/>
     </row>
-    <row r="10" spans="10:74" x14ac:dyDescent="0.2">
+    <row r="10" spans="10:74" x14ac:dyDescent="0.25">
       <c r="J10" s="2"/>
       <c r="Q10">
         <v>7</v>
@@ -3500,14 +3491,13 @@
       <c r="S10">
         <v>-1</v>
       </c>
-      <c r="Z10" s="14"/>
-      <c r="AA10" s="5"/>
-      <c r="AB10" s="12"/>
-      <c r="AC10" s="12"/>
-      <c r="AD10" s="12"/>
-      <c r="AE10" s="12"/>
-      <c r="AF10" s="12"/>
-      <c r="AG10" s="13"/>
+      <c r="Z10" s="4"/>
+      <c r="AB10" s="10"/>
+      <c r="AC10" s="10"/>
+      <c r="AD10" s="10"/>
+      <c r="AE10" s="10"/>
+      <c r="AF10" s="10"/>
+      <c r="AG10" s="11"/>
       <c r="AJ10">
         <v>7</v>
       </c>
@@ -3533,24 +3523,23 @@
         <v>7</v>
       </c>
       <c r="BA10">
+        <v>9</v>
+      </c>
+      <c r="BB10">
         <v>6</v>
       </c>
-      <c r="BB10">
+      <c r="BC10">
         <v>7</v>
       </c>
-      <c r="BC10">
-        <v>9</v>
-      </c>
-      <c r="BO10" s="14"/>
-      <c r="BP10" s="5"/>
-      <c r="BQ10" s="12"/>
-      <c r="BR10" s="12"/>
-      <c r="BS10" s="12"/>
-      <c r="BT10" s="12"/>
-      <c r="BU10" s="12"/>
-      <c r="BV10" s="13"/>
+      <c r="BO10" s="4"/>
+      <c r="BQ10" s="10"/>
+      <c r="BR10" s="10"/>
+      <c r="BS10" s="10"/>
+      <c r="BT10" s="10"/>
+      <c r="BU10" s="10"/>
+      <c r="BV10" s="11"/>
     </row>
-    <row r="11" spans="10:74" x14ac:dyDescent="0.2">
+    <row r="11" spans="10:74" x14ac:dyDescent="0.25">
       <c r="Q11">
         <v>8</v>
       </c>
@@ -3560,8 +3549,8 @@
       <c r="S11">
         <v>-4</v>
       </c>
-      <c r="Z11" s="14"/>
-      <c r="AA11" s="15"/>
+      <c r="Z11" s="4"/>
+      <c r="AA11" s="12"/>
       <c r="AJ11">
         <v>8</v>
       </c>
@@ -3587,18 +3576,18 @@
         <v>8</v>
       </c>
       <c r="BA11">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="BB11">
         <v>8</v>
       </c>
       <c r="BC11">
-        <v>11</v>
-      </c>
-      <c r="BO11" s="14"/>
-      <c r="BP11" s="15"/>
+        <v>10</v>
+      </c>
+      <c r="BO11" s="4"/>
+      <c r="BP11" s="12"/>
     </row>
-    <row r="12" spans="10:74" x14ac:dyDescent="0.2">
+    <row r="12" spans="10:74" x14ac:dyDescent="0.25">
       <c r="Q12">
         <v>9</v>
       </c>
@@ -3608,8 +3597,8 @@
       <c r="S12">
         <v>-4</v>
       </c>
-      <c r="Z12" s="14"/>
-      <c r="AA12" s="15"/>
+      <c r="Z12" s="4"/>
+      <c r="AA12" s="12"/>
       <c r="AJ12">
         <v>9</v>
       </c>
@@ -3631,24 +3620,12 @@
       <c r="AV12">
         <v>1</v>
       </c>
-      <c r="AZ12">
-        <v>9</v>
-      </c>
-      <c r="BA12">
-        <v>4</v>
-      </c>
-      <c r="BB12">
-        <v>2</v>
-      </c>
-      <c r="BC12">
-        <v>1</v>
-      </c>
-      <c r="BO12" s="14"/>
-      <c r="BP12" s="15"/>
+      <c r="BO12" s="4"/>
+      <c r="BP12" s="12"/>
     </row>
-    <row r="13" spans="10:74" x14ac:dyDescent="0.2">
-      <c r="Z13" s="14"/>
-      <c r="AA13" s="15"/>
+    <row r="13" spans="10:74" x14ac:dyDescent="0.25">
+      <c r="Z13" s="4"/>
+      <c r="AA13" s="12"/>
       <c r="AJ13">
         <v>10</v>
       </c>
@@ -3671,23 +3648,23 @@
         <v>1</v>
       </c>
       <c r="AZ13">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="BA13">
+        <v>1</v>
+      </c>
+      <c r="BB13">
+        <v>2</v>
+      </c>
+      <c r="BC13">
         <v>4</v>
       </c>
-      <c r="BB13">
-        <v>1</v>
-      </c>
-      <c r="BC13">
-        <v>3</v>
-      </c>
-      <c r="BO13" s="14"/>
-      <c r="BP13" s="15"/>
+      <c r="BO13" s="4"/>
+      <c r="BP13" s="12"/>
     </row>
-    <row r="14" spans="10:74" x14ac:dyDescent="0.2">
-      <c r="Z14" s="14"/>
-      <c r="AA14" s="15"/>
+    <row r="14" spans="10:74" x14ac:dyDescent="0.25">
+      <c r="Z14" s="4"/>
+      <c r="AA14" s="12"/>
       <c r="AJ14">
         <v>11</v>
       </c>
@@ -3710,24 +3687,23 @@
         <v>1</v>
       </c>
       <c r="AZ14">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="BA14">
+        <v>3</v>
+      </c>
+      <c r="BB14">
         <v>1</v>
       </c>
-      <c r="BB14">
-        <v>0</v>
-      </c>
       <c r="BC14">
-        <v>3</v>
-      </c>
-      <c r="BO14" s="14"/>
-      <c r="BP14" s="15"/>
-      <c r="BV14" s="5"/>
+        <v>4</v>
+      </c>
+      <c r="BO14" s="4"/>
+      <c r="BP14" s="12"/>
     </row>
-    <row r="15" spans="10:74" x14ac:dyDescent="0.2">
-      <c r="Z15" s="14"/>
-      <c r="AA15" s="15"/>
+    <row r="15" spans="10:74" x14ac:dyDescent="0.25">
+      <c r="Z15" s="4"/>
+      <c r="AA15" s="12"/>
       <c r="AS15">
         <v>0</v>
       </c>
@@ -3741,29 +3717,28 @@
         <v>-1</v>
       </c>
       <c r="AZ15">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="BA15">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="BB15">
+        <v>1</v>
+      </c>
+      <c r="BC15">
         <v>3</v>
       </c>
-      <c r="BC15">
-        <v>0</v>
-      </c>
-      <c r="BO15" s="14"/>
-      <c r="BP15" s="5"/>
-      <c r="BQ15" s="10"/>
-      <c r="BR15" s="10"/>
-      <c r="BS15" s="10"/>
-      <c r="BT15" s="10"/>
-      <c r="BU15" s="10"/>
-      <c r="BV15" s="16"/>
+      <c r="BO15" s="4"/>
+      <c r="BQ15" s="8"/>
+      <c r="BR15" s="8"/>
+      <c r="BS15" s="8"/>
+      <c r="BT15" s="8"/>
+      <c r="BU15" s="8"/>
+      <c r="BV15" s="13"/>
     </row>
-    <row r="16" spans="10:74" x14ac:dyDescent="0.2">
-      <c r="Z16" s="14"/>
-      <c r="AA16" s="15"/>
+    <row r="16" spans="10:74" x14ac:dyDescent="0.25">
+      <c r="Z16" s="4"/>
+      <c r="AA16" s="12"/>
       <c r="AS16">
         <v>1</v>
       </c>
@@ -3777,29 +3752,28 @@
         <v>-1</v>
       </c>
       <c r="AZ16">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="BA16">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BB16">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="BC16">
         <v>8</v>
       </c>
-      <c r="BO16" s="14"/>
-      <c r="BP16" s="5"/>
-      <c r="BQ16" s="12"/>
-      <c r="BR16" s="12"/>
-      <c r="BS16" s="12"/>
-      <c r="BT16" s="12"/>
-      <c r="BU16" s="12"/>
-      <c r="BV16" s="13"/>
+      <c r="BO16" s="4"/>
+      <c r="BQ16" s="10"/>
+      <c r="BR16" s="10"/>
+      <c r="BS16" s="10"/>
+      <c r="BT16" s="10"/>
+      <c r="BU16" s="10"/>
+      <c r="BV16" s="11"/>
     </row>
-    <row r="17" spans="26:76" x14ac:dyDescent="0.2">
-      <c r="Z17" s="14"/>
-      <c r="AA17" s="15"/>
+    <row r="17" spans="26:68" x14ac:dyDescent="0.25">
+      <c r="Z17" s="4"/>
+      <c r="AA17" s="12"/>
       <c r="AS17">
         <v>2</v>
       </c>
@@ -3813,23 +3787,23 @@
         <v>-1</v>
       </c>
       <c r="AZ17">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="BA17">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="BB17">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="BC17">
-        <v>8</v>
-      </c>
-      <c r="BO17" s="14"/>
-      <c r="BP17" s="15"/>
+        <v>10</v>
+      </c>
+      <c r="BO17" s="4"/>
+      <c r="BP17" s="12"/>
     </row>
-    <row r="18" spans="26:76" x14ac:dyDescent="0.2">
-      <c r="Z18" s="11"/>
-      <c r="AA18" s="13"/>
+    <row r="18" spans="26:68" x14ac:dyDescent="0.25">
+      <c r="Z18" s="9"/>
+      <c r="AA18" s="11"/>
       <c r="AS18">
         <v>3</v>
       </c>
@@ -3843,21 +3817,21 @@
         <v>-1</v>
       </c>
       <c r="AZ18">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="BA18">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="BB18">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="BC18">
         <v>6</v>
       </c>
-      <c r="BO18" s="14"/>
-      <c r="BP18" s="15"/>
+      <c r="BO18" s="4"/>
+      <c r="BP18" s="12"/>
     </row>
-    <row r="19" spans="26:76" x14ac:dyDescent="0.2">
+    <row r="19" spans="26:68" x14ac:dyDescent="0.25">
       <c r="AS19">
         <v>4</v>
       </c>
@@ -3871,21 +3845,21 @@
         <v>-1</v>
       </c>
       <c r="AZ19">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="BA19">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="BB19">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="BC19">
-        <v>11</v>
-      </c>
-      <c r="BO19" s="14"/>
-      <c r="BP19" s="15"/>
+        <v>9</v>
+      </c>
+      <c r="BO19" s="4"/>
+      <c r="BP19" s="12"/>
     </row>
-    <row r="20" spans="26:76" x14ac:dyDescent="0.2">
+    <row r="20" spans="26:68" x14ac:dyDescent="0.25">
       <c r="AS20">
         <v>5</v>
       </c>
@@ -3898,10 +3872,22 @@
       <c r="AV20">
         <v>-1</v>
       </c>
-      <c r="BO20" s="14"/>
-      <c r="BP20" s="15"/>
+      <c r="AZ20">
+        <v>16</v>
+      </c>
+      <c r="BA20">
+        <v>6</v>
+      </c>
+      <c r="BB20">
+        <v>7</v>
+      </c>
+      <c r="BC20">
+        <v>9</v>
+      </c>
+      <c r="BO20" s="4"/>
+      <c r="BP20" s="12"/>
     </row>
-    <row r="21" spans="26:76" x14ac:dyDescent="0.2">
+    <row r="21" spans="26:68" x14ac:dyDescent="0.25">
       <c r="AS21">
         <v>6</v>
       </c>
@@ -3914,10 +3900,22 @@
       <c r="AV21">
         <v>-1</v>
       </c>
-      <c r="BO21" s="14"/>
-      <c r="BP21" s="15"/>
+      <c r="AZ21">
+        <v>17</v>
+      </c>
+      <c r="BA21">
+        <v>10</v>
+      </c>
+      <c r="BB21">
+        <v>8</v>
+      </c>
+      <c r="BC21">
+        <v>11</v>
+      </c>
+      <c r="BO21" s="4"/>
+      <c r="BP21" s="12"/>
     </row>
-    <row r="22" spans="26:76" x14ac:dyDescent="0.2">
+    <row r="22" spans="26:68" x14ac:dyDescent="0.25">
       <c r="AS22">
         <v>7</v>
       </c>
@@ -3930,10 +3928,10 @@
       <c r="AV22">
         <v>-1</v>
       </c>
-      <c r="BO22" s="14"/>
-      <c r="BP22" s="15"/>
+      <c r="BO22" s="4"/>
+      <c r="BP22" s="12"/>
     </row>
-    <row r="23" spans="26:76" x14ac:dyDescent="0.2">
+    <row r="23" spans="26:68" x14ac:dyDescent="0.25">
       <c r="AS23">
         <v>8</v>
       </c>
@@ -3946,10 +3944,10 @@
       <c r="AV23">
         <v>-1</v>
       </c>
-      <c r="BO23" s="14"/>
-      <c r="BP23" s="15"/>
+      <c r="BO23" s="4"/>
+      <c r="BP23" s="12"/>
     </row>
-    <row r="24" spans="26:76" x14ac:dyDescent="0.2">
+    <row r="24" spans="26:68" x14ac:dyDescent="0.25">
       <c r="AS24">
         <v>9</v>
       </c>
@@ -3962,10 +3960,10 @@
       <c r="AV24">
         <v>-1</v>
       </c>
-      <c r="BO24" s="11"/>
-      <c r="BP24" s="13"/>
+      <c r="BO24" s="9"/>
+      <c r="BP24" s="11"/>
     </row>
-    <row r="25" spans="26:76" x14ac:dyDescent="0.2">
+    <row r="25" spans="26:68" x14ac:dyDescent="0.25">
       <c r="AS25">
         <v>10</v>
       </c>
@@ -3979,7 +3977,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="26" spans="26:76" x14ac:dyDescent="0.2">
+    <row r="26" spans="26:68" x14ac:dyDescent="0.25">
       <c r="AS26">
         <v>11</v>
       </c>
@@ -3992,7 +3990,6 @@
       <c r="AV26">
         <v>-1</v>
       </c>
-      <c r="BX26" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>